<commit_message>
feat(works): 新增 thumb_url/backdrop_url/score 富字段（ADR-0002）
metatube adapter 此前静默丢弃 MovieInfo 的高价值字段，本次按 ADR-0002 落库：
- works.schema.json 新增 thumb_url/backdrop_url/score 三列（cover_url 之后）
- metatube adapter 映射 summary→description、thumb_url、backdrop_url、score
- import 管线 WORK_OBSERVABLE_FIELDS 纳入新字段，使 Phase 4 观察/裁决覆盖评分
- data/works/works.csv 列迁移，既有数据无损；重新生成 json/xlsx 导出
</commit_message>
<xml_diff>
--- a/exports/xlsx/averia.xlsx
+++ b/exports/xlsx/averia.xlsx
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="361" uniqueCount="151">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="364" uniqueCount="154">
   <si>
     <t>女优ID</t>
   </si>
@@ -259,6 +259,15 @@
   </si>
   <si>
     <t>系列ID</t>
+  </si>
+  <si>
+    <t>缩略图URL</t>
+  </si>
+  <si>
+    <t>背景图URL</t>
+  </si>
+  <si>
+    <t>评分</t>
   </si>
   <si>
     <t>maker_000001</t>
@@ -1088,13 +1097,13 @@
         <v>75</v>
       </c>
       <c r="B1" s="5" t="s">
-        <v>107</v>
+        <v>110</v>
       </c>
       <c r="C1" s="5" t="s">
         <v>2</v>
       </c>
       <c r="D1" s="5" t="s">
-        <v>108</v>
+        <v>111</v>
       </c>
       <c r="E1" s="5" t="s">
         <v>16</v>
@@ -1108,7 +1117,7 @@
     </row>
     <row r="2" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A2" s="3" t="s">
-        <v>78</v>
+        <v>81</v>
       </c>
       <c r="B2" s="3" t="s">
         <v>47</v>
@@ -1117,7 +1126,7 @@
         <v>47</v>
       </c>
       <c r="D2" s="3" t="s">
-        <v>109</v>
+        <v>112</v>
       </c>
       <c r="E2" s="3"/>
       <c r="F2" s="3" t="s">
@@ -1129,7 +1138,7 @@
     </row>
     <row r="3" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A3" s="3" t="s">
-        <v>81</v>
+        <v>84</v>
       </c>
       <c r="B3" s="3" t="s">
         <v>56</v>
@@ -1170,13 +1179,13 @@
         <v>75</v>
       </c>
       <c r="C1" s="5" t="s">
-        <v>107</v>
+        <v>110</v>
       </c>
       <c r="D1" s="5" t="s">
         <v>2</v>
       </c>
       <c r="E1" s="5" t="s">
-        <v>108</v>
+        <v>111</v>
       </c>
       <c r="F1" s="5" t="s">
         <v>16</v>
@@ -1190,10 +1199,10 @@
     </row>
     <row r="2" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A2" s="3" t="s">
-        <v>79</v>
+        <v>82</v>
       </c>
       <c r="B2" s="3" t="s">
-        <v>78</v>
+        <v>81</v>
       </c>
       <c r="C2" s="3" t="s">
         <v>48</v>
@@ -1212,10 +1221,10 @@
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A3" s="3" t="s">
-        <v>82</v>
+        <v>85</v>
       </c>
       <c r="B3" s="3" t="s">
-        <v>81</v>
+        <v>84</v>
       </c>
       <c r="C3" s="3" t="s">
         <v>57</v>
@@ -1256,7 +1265,7 @@
         <v>76</v>
       </c>
       <c r="D1" s="5" t="s">
-        <v>107</v>
+        <v>110</v>
       </c>
       <c r="E1" s="5" t="s">
         <v>2</v>
@@ -1292,19 +1301,19 @@
   <sheetData>
     <row r="1" ht="24" customHeight="1" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="5" t="s">
-        <v>97</v>
+        <v>100</v>
       </c>
       <c r="B1" s="5" t="s">
-        <v>107</v>
+        <v>110</v>
       </c>
       <c r="C1" s="5" t="s">
         <v>2</v>
       </c>
       <c r="D1" s="5" t="s">
-        <v>110</v>
+        <v>113</v>
       </c>
       <c r="E1" s="5" t="s">
-        <v>111</v>
+        <v>114</v>
       </c>
       <c r="F1" s="5" t="s">
         <v>63</v>
@@ -1315,16 +1324,16 @@
     </row>
     <row r="2" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A2" s="3" t="s">
-        <v>98</v>
+        <v>101</v>
       </c>
       <c r="B2" s="3" t="s">
-        <v>112</v>
+        <v>115</v>
       </c>
       <c r="C2" s="3" t="s">
-        <v>112</v>
+        <v>115</v>
       </c>
       <c r="D2" s="3" t="s">
-        <v>113</v>
+        <v>116</v>
       </c>
       <c r="E2" s="3"/>
       <c r="F2" s="3" t="s">
@@ -1336,16 +1345,16 @@
     </row>
     <row r="3" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A3" s="3" t="s">
-        <v>99</v>
+        <v>102</v>
       </c>
       <c r="B3" s="3" t="s">
-        <v>114</v>
+        <v>117</v>
       </c>
       <c r="C3" s="3" t="s">
-        <v>114</v>
+        <v>117</v>
       </c>
       <c r="D3" s="3" t="s">
-        <v>115</v>
+        <v>118</v>
       </c>
       <c r="E3" s="3"/>
       <c r="F3" s="3" t="s">
@@ -1357,16 +1366,16 @@
     </row>
     <row r="4" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A4" s="3" t="s">
-        <v>100</v>
+        <v>103</v>
       </c>
       <c r="B4" s="3" t="s">
-        <v>116</v>
+        <v>119</v>
       </c>
       <c r="C4" s="3" t="s">
-        <v>116</v>
+        <v>119</v>
       </c>
       <c r="D4" s="3" t="s">
-        <v>117</v>
+        <v>120</v>
       </c>
       <c r="E4" s="3"/>
       <c r="F4" s="3" t="s">
@@ -1378,16 +1387,16 @@
     </row>
     <row r="5" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A5" s="3" t="s">
-        <v>101</v>
+        <v>104</v>
       </c>
       <c r="B5" s="3" t="s">
-        <v>118</v>
+        <v>121</v>
       </c>
       <c r="C5" s="3" t="s">
-        <v>118</v>
+        <v>121</v>
       </c>
       <c r="D5" s="3" t="s">
-        <v>119</v>
+        <v>122</v>
       </c>
       <c r="E5" s="3"/>
       <c r="F5" s="3" t="s">
@@ -1399,16 +1408,16 @@
     </row>
     <row r="6" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A6" s="3" t="s">
-        <v>102</v>
+        <v>105</v>
       </c>
       <c r="B6" s="3" t="s">
-        <v>120</v>
+        <v>123</v>
       </c>
       <c r="C6" s="3" t="s">
-        <v>120</v>
+        <v>123</v>
       </c>
       <c r="D6" s="3" t="s">
-        <v>121</v>
+        <v>124</v>
       </c>
       <c r="E6" s="3"/>
       <c r="F6" s="3" t="s">
@@ -1420,16 +1429,16 @@
     </row>
     <row r="7" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A7" s="3" t="s">
-        <v>103</v>
+        <v>106</v>
       </c>
       <c r="B7" s="3" t="s">
-        <v>122</v>
+        <v>125</v>
       </c>
       <c r="C7" s="3" t="s">
-        <v>122</v>
+        <v>125</v>
       </c>
       <c r="D7" s="3" t="s">
-        <v>123</v>
+        <v>126</v>
       </c>
       <c r="E7" s="3"/>
       <c r="F7" s="3" t="s">
@@ -1441,14 +1450,14 @@
     </row>
     <row r="8" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A8" s="3" t="s">
-        <v>104</v>
+        <v>107</v>
       </c>
       <c r="B8" s="3" t="s">
         <v>58</v>
       </c>
       <c r="C8" s="3"/>
       <c r="D8" s="3" t="s">
-        <v>124</v>
+        <v>127</v>
       </c>
       <c r="E8" s="3"/>
       <c r="F8" s="3" t="s">
@@ -1477,16 +1486,16 @@
   <sheetData>
     <row r="1" ht="24" customHeight="1" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="5" t="s">
-        <v>105</v>
+        <v>108</v>
       </c>
       <c r="B1" s="5" t="s">
-        <v>107</v>
+        <v>110</v>
       </c>
       <c r="C1" s="5" t="s">
         <v>2</v>
       </c>
       <c r="D1" s="5" t="s">
-        <v>108</v>
+        <v>111</v>
       </c>
       <c r="E1" s="5" t="s">
         <v>16</v>
@@ -1500,7 +1509,7 @@
     </row>
     <row r="2" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A2" s="3" t="s">
-        <v>106</v>
+        <v>109</v>
       </c>
       <c r="B2" s="3" t="s">
         <v>49</v>
@@ -1545,131 +1554,131 @@
         <v>69</v>
       </c>
       <c r="B1" s="5" t="s">
-        <v>125</v>
+        <v>128</v>
       </c>
       <c r="C1" s="5" t="s">
-        <v>126</v>
+        <v>129</v>
       </c>
       <c r="D1" s="5" t="s">
-        <v>127</v>
+        <v>130</v>
       </c>
       <c r="E1" s="5" t="s">
-        <v>128</v>
+        <v>131</v>
       </c>
       <c r="F1" s="5" t="s">
-        <v>129</v>
+        <v>132</v>
       </c>
       <c r="G1" s="5" t="s">
-        <v>130</v>
+        <v>133</v>
       </c>
       <c r="H1" s="5" t="s">
-        <v>131</v>
+        <v>134</v>
       </c>
       <c r="I1" s="5" t="s">
-        <v>132</v>
+        <v>135</v>
       </c>
     </row>
     <row r="2" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A2" s="3" t="s">
-        <v>133</v>
+        <v>136</v>
       </c>
       <c r="B2" s="3" t="s">
-        <v>96</v>
+        <v>99</v>
       </c>
       <c r="C2" s="3" t="s">
         <v>18</v>
       </c>
       <c r="D2" s="3" t="s">
-        <v>134</v>
+        <v>137</v>
       </c>
       <c r="E2" s="3" t="s">
-        <v>135</v>
+        <v>138</v>
       </c>
       <c r="F2" s="3" t="s">
-        <v>136</v>
+        <v>139</v>
       </c>
       <c r="G2" s="3" t="s">
-        <v>137</v>
+        <v>140</v>
       </c>
       <c r="H2" s="3" t="s">
-        <v>138</v>
+        <v>141</v>
       </c>
       <c r="I2" s="3"/>
     </row>
     <row r="3" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A3" s="3" t="s">
-        <v>90</v>
+        <v>93</v>
       </c>
       <c r="B3" s="3" t="s">
-        <v>139</v>
+        <v>142</v>
       </c>
       <c r="C3" s="3" t="s">
         <v>43</v>
       </c>
       <c r="D3" s="3" t="s">
-        <v>134</v>
+        <v>137</v>
       </c>
       <c r="E3" s="3" t="s">
-        <v>140</v>
+        <v>143</v>
       </c>
       <c r="F3" s="3" t="s">
-        <v>141</v>
+        <v>144</v>
       </c>
       <c r="G3" s="3" t="s">
-        <v>142</v>
+        <v>145</v>
       </c>
       <c r="H3" s="3" t="s">
-        <v>143</v>
+        <v>146</v>
       </c>
       <c r="I3" s="3"/>
     </row>
     <row r="4" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A4" s="3" t="s">
-        <v>144</v>
+        <v>147</v>
       </c>
       <c r="B4" s="3" t="s">
-        <v>96</v>
+        <v>99</v>
       </c>
       <c r="C4" s="3" t="s">
         <v>27</v>
       </c>
       <c r="D4" s="3" t="s">
-        <v>145</v>
+        <v>148</v>
       </c>
       <c r="E4" s="3" t="s">
-        <v>146</v>
+        <v>149</v>
       </c>
       <c r="F4" s="3"/>
       <c r="G4" s="3" t="s">
-        <v>147</v>
+        <v>150</v>
       </c>
       <c r="H4" s="3" t="s">
-        <v>148</v>
+        <v>151</v>
       </c>
       <c r="I4" s="3"/>
     </row>
     <row r="5" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A5" s="3" t="s">
-        <v>93</v>
+        <v>96</v>
       </c>
       <c r="B5" s="3" t="s">
-        <v>139</v>
+        <v>142</v>
       </c>
       <c r="C5" s="3" t="s">
         <v>52</v>
       </c>
       <c r="D5" s="3" t="s">
-        <v>145</v>
+        <v>148</v>
       </c>
       <c r="E5" s="3" t="s">
-        <v>149</v>
+        <v>152</v>
       </c>
       <c r="F5" s="3"/>
       <c r="G5" s="3" t="s">
-        <v>147</v>
+        <v>150</v>
       </c>
       <c r="H5" s="3" t="s">
-        <v>150</v>
+        <v>153</v>
       </c>
       <c r="I5" s="3"/>
     </row>
@@ -2066,7 +2075,7 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:M3"/>
+  <dimension ref="A1:P3"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="15" customWidth="1"/>
@@ -2077,10 +2086,11 @@
     <col min="7" max="8" width="16" customWidth="1"/>
     <col min="9" max="10" width="12" customWidth="1"/>
     <col min="11" max="11" width="40" customWidth="1"/>
-    <col min="12" max="13" width="24" customWidth="1"/>
+    <col min="12" max="14" width="12" customWidth="1"/>
+    <col min="15" max="16" width="24" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" ht="24" customHeight="1" spans="1:13" s="4" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="1" ht="24" customHeight="1" spans="1:16" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="5" t="s">
         <v>31</v>
       </c>
@@ -2115,13 +2125,22 @@
         <v>42</v>
       </c>
       <c r="L1" s="5" t="s">
+        <v>78</v>
+      </c>
+      <c r="M1" s="5" t="s">
+        <v>79</v>
+      </c>
+      <c r="N1" s="5" t="s">
+        <v>80</v>
+      </c>
+      <c r="O1" s="5" t="s">
         <v>63</v>
       </c>
-      <c r="M1" s="5" t="s">
+      <c r="P1" s="5" t="s">
         <v>17</v>
       </c>
     </row>
-    <row r="2" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A2" s="3" t="s">
         <v>43</v>
       </c>
@@ -2141,24 +2160,27 @@
         <v>90</v>
       </c>
       <c r="G2" s="3" t="s">
-        <v>78</v>
+        <v>81</v>
       </c>
       <c r="H2" s="3" t="s">
-        <v>79</v>
+        <v>82</v>
       </c>
       <c r="I2" s="3"/>
       <c r="J2" s="3"/>
       <c r="K2" s="3" t="s">
         <v>51</v>
       </c>
-      <c r="L2" s="3" t="s">
+      <c r="L2" s="3"/>
+      <c r="M2" s="3"/>
+      <c r="N2" s="3"/>
+      <c r="O2" s="3" t="s">
         <v>26</v>
       </c>
-      <c r="M2" s="3" t="s">
+      <c r="P2" s="3" t="s">
         <v>26</v>
       </c>
     </row>
-    <row r="3" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A3" s="3" t="s">
         <v>52</v>
       </c>
@@ -2166,7 +2188,7 @@
         <v>53</v>
       </c>
       <c r="C3" s="3" t="s">
-        <v>80</v>
+        <v>83</v>
       </c>
       <c r="D3" s="3" t="s">
         <v>54</v>
@@ -2178,23 +2200,26 @@
         <v>127</v>
       </c>
       <c r="G3" s="3" t="s">
-        <v>81</v>
+        <v>84</v>
       </c>
       <c r="H3" s="3" t="s">
-        <v>82</v>
+        <v>85</v>
       </c>
       <c r="I3" s="3"/>
       <c r="J3" s="3"/>
       <c r="K3" s="3"/>
-      <c r="L3" s="3" t="s">
+      <c r="L3" s="3"/>
+      <c r="M3" s="3"/>
+      <c r="N3" s="3"/>
+      <c r="O3" s="3" t="s">
         <v>30</v>
       </c>
-      <c r="M3" s="3" t="s">
+      <c r="P3" s="3" t="s">
         <v>30</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:M3"/>
+  <autoFilter ref="A1:P3"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
 </worksheet>
@@ -2212,7 +2237,7 @@
   <sheetData>
     <row r="1" ht="24" customHeight="1" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="5" t="s">
-        <v>83</v>
+        <v>86</v>
       </c>
       <c r="B1" s="5" t="s">
         <v>31</v>
@@ -2221,13 +2246,13 @@
         <v>32</v>
       </c>
       <c r="D1" s="5" t="s">
-        <v>84</v>
+        <v>87</v>
       </c>
       <c r="E1" s="5" t="s">
-        <v>85</v>
+        <v>88</v>
       </c>
       <c r="F1" s="5" t="s">
-        <v>86</v>
+        <v>89</v>
       </c>
       <c r="G1" s="5" t="s">
         <v>69</v>
@@ -2235,7 +2260,7 @@
     </row>
     <row r="2" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A2" s="3" t="s">
-        <v>87</v>
+        <v>90</v>
       </c>
       <c r="B2" s="3" t="s">
         <v>43</v>
@@ -2244,21 +2269,21 @@
         <v>44</v>
       </c>
       <c r="D2" s="3" t="s">
-        <v>88</v>
+        <v>91</v>
       </c>
       <c r="E2" s="3" t="s">
-        <v>89</v>
+        <v>92</v>
       </c>
       <c r="F2" s="3" t="b">
         <v>1</v>
       </c>
       <c r="G2" s="3" t="s">
-        <v>90</v>
+        <v>93</v>
       </c>
     </row>
     <row r="3" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A3" s="3" t="s">
-        <v>91</v>
+        <v>94</v>
       </c>
       <c r="B3" s="3" t="s">
         <v>52</v>
@@ -2267,16 +2292,16 @@
         <v>53</v>
       </c>
       <c r="D3" s="3" t="s">
+        <v>95</v>
+      </c>
+      <c r="E3" s="3" t="s">
         <v>92</v>
-      </c>
-      <c r="E3" s="3" t="s">
-        <v>89</v>
       </c>
       <c r="F3" s="3" t="b">
         <v>1</v>
       </c>
       <c r="G3" s="3" t="s">
-        <v>93</v>
+        <v>96</v>
       </c>
     </row>
   </sheetData>
@@ -2304,10 +2329,10 @@
         <v>0</v>
       </c>
       <c r="C1" s="5" t="s">
-        <v>94</v>
+        <v>97</v>
       </c>
       <c r="D1" s="5" t="s">
-        <v>95</v>
+        <v>98</v>
       </c>
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.25">
@@ -2318,7 +2343,7 @@
         <v>18</v>
       </c>
       <c r="C2" s="3" t="s">
-        <v>96</v>
+        <v>99</v>
       </c>
       <c r="D2" s="3">
         <v>1</v>
@@ -2332,7 +2357,7 @@
         <v>27</v>
       </c>
       <c r="C3" s="3" t="s">
-        <v>96</v>
+        <v>99</v>
       </c>
       <c r="D3" s="3">
         <v>1</v>
@@ -2359,7 +2384,7 @@
         <v>31</v>
       </c>
       <c r="B1" s="5" t="s">
-        <v>97</v>
+        <v>100</v>
       </c>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.25">
@@ -2367,7 +2392,7 @@
         <v>43</v>
       </c>
       <c r="B2" s="3" t="s">
-        <v>98</v>
+        <v>101</v>
       </c>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.25">
@@ -2375,7 +2400,7 @@
         <v>43</v>
       </c>
       <c r="B3" s="3" t="s">
-        <v>99</v>
+        <v>102</v>
       </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.25">
@@ -2383,7 +2408,7 @@
         <v>43</v>
       </c>
       <c r="B4" s="3" t="s">
-        <v>100</v>
+        <v>103</v>
       </c>
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.25">
@@ -2391,7 +2416,7 @@
         <v>43</v>
       </c>
       <c r="B5" s="3" t="s">
-        <v>101</v>
+        <v>104</v>
       </c>
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.25">
@@ -2399,7 +2424,7 @@
         <v>43</v>
       </c>
       <c r="B6" s="3" t="s">
-        <v>102</v>
+        <v>105</v>
       </c>
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.25">
@@ -2407,7 +2432,7 @@
         <v>43</v>
       </c>
       <c r="B7" s="3" t="s">
-        <v>103</v>
+        <v>106</v>
       </c>
     </row>
     <row r="8" spans="1:2" x14ac:dyDescent="0.25">
@@ -2415,7 +2440,7 @@
         <v>52</v>
       </c>
       <c r="B8" s="3" t="s">
-        <v>104</v>
+        <v>107</v>
       </c>
     </row>
   </sheetData>
@@ -2440,10 +2465,10 @@
         <v>31</v>
       </c>
       <c r="B1" s="5" t="s">
-        <v>105</v>
+        <v>108</v>
       </c>
       <c r="C1" s="5" t="s">
-        <v>95</v>
+        <v>98</v>
       </c>
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.25">
@@ -2451,7 +2476,7 @@
         <v>43</v>
       </c>
       <c r="B2" s="3" t="s">
-        <v>106</v>
+        <v>109</v>
       </c>
       <c r="C2" s="3">
         <v>1</v>

</xml_diff>

<commit_message>
data(ingest): 经 MetaTube 灌入 4 部 javbus 作品及分类/关系
通过本地 metatube-server（v1.4.0 Windows 二进制）+ scripts/ingest-metatube.mjs
批量灌库，新增 4 部作品（SSIS-001/MIDE-345/IPX-001/WANZ-912）及其 5 位女优，
并完整物化 taxonomy（makers/labels/series/genres/directors）与 relations
（work_cast/work_genres/work_directors）关联表，共 +207 行数据。
同步重新生成 exports/json、exports/xlsx。
</commit_message>
<xml_diff>
--- a/exports/xlsx/averia.xlsx
+++ b/exports/xlsx/averia.xlsx
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="364" uniqueCount="154">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="892" uniqueCount="305">
   <si>
     <t>女优ID</t>
   </si>
@@ -120,6 +120,39 @@
     <t>2026-09-04T06:26:39Z</t>
   </si>
   <si>
+    <t>actress_000003</t>
+  </si>
+  <si>
+    <t>葵つかさ</t>
+  </si>
+  <si>
+    <t>2026-09-04T08:56:42Z</t>
+  </si>
+  <si>
+    <t>actress_000004</t>
+  </si>
+  <si>
+    <t>乙白さやか</t>
+  </si>
+  <si>
+    <t>actress_000005</t>
+  </si>
+  <si>
+    <t>JULIA</t>
+  </si>
+  <si>
+    <t>actress_000006</t>
+  </si>
+  <si>
+    <t>妃月るい</t>
+  </si>
+  <si>
+    <t>actress_000007</t>
+  </si>
+  <si>
+    <t>桐谷まつり</t>
+  </si>
+  <si>
     <t>作品ID</t>
   </si>
   <si>
@@ -204,6 +237,111 @@
     <t>Slender</t>
   </si>
   <si>
+    <t>work_000003</t>
+  </si>
+  <si>
+    <t>SSIS-001</t>
+  </si>
+  <si>
+    <t>一ヶ月間の禁欲の果てに彼女のルームメイト2人と浮気SEXだけに没頭した彼女不在の3日間。 葵つかさ 乙白さやか</t>
+  </si>
+  <si>
+    <t>葵つかさ、乙白さやか</t>
+  </si>
+  <si>
+    <t>2021-02-18</t>
+  </si>
+  <si>
+    <t>エスワン ナンバーワンスタイル</t>
+  </si>
+  <si>
+    <t>S1 NO.1 STYLE</t>
+  </si>
+  <si>
+    <t>苺原</t>
+  </si>
+  <si>
+    <t>3P・4P、美少女、美乳、ギリモザ、ハイビジョン、寝取り・寝取られ、ドラマ、独占配信</t>
+  </si>
+  <si>
+    <t>https://www.javbus.com/pics/cover/83ie_b.jpg</t>
+  </si>
+  <si>
+    <t>work_000004</t>
+  </si>
+  <si>
+    <t>MIDE-345</t>
+  </si>
+  <si>
+    <t>JULIA 騎乗位SPECIAL</t>
+  </si>
+  <si>
+    <t>2016-07-30</t>
+  </si>
+  <si>
+    <t>ムーディーズ</t>
+  </si>
+  <si>
+    <t>MOODYZDIVA</t>
+  </si>
+  <si>
+    <t>南★波王</t>
+  </si>
+  <si>
+    <t>淫語、デジモ、騎乗位、主観、ハイビジョン、顔面騎乗、巨乳、単体作品、独占配信</t>
+  </si>
+  <si>
+    <t>https://www.javbus.com/pics/cover/5klt_b.jpg</t>
+  </si>
+  <si>
+    <t>work_000005</t>
+  </si>
+  <si>
+    <t>IPX-001</t>
+  </si>
+  <si>
+    <t>女子校生便所交際 便所でしか濡れないおじさん好きの変態マゾ美少女と思う存分便所ファック！ 妃月るい</t>
+  </si>
+  <si>
+    <t>2017-08-11</t>
+  </si>
+  <si>
+    <t>刃修羅</t>
+  </si>
+  <si>
+    <t>ハメ撮り、美少女、デジモ、イラマチオ、ハイビジョン、女子校生、巨乳、単体作品、独占配信</t>
+  </si>
+  <si>
+    <t>https://www.javbus.com/pics/cover/649d_b.jpg</t>
+  </si>
+  <si>
+    <t>work_000006</t>
+  </si>
+  <si>
+    <t>WANZ-912</t>
+  </si>
+  <si>
+    <t>男潮吹きそのまま挿入、スプラッシュ中出し！ 桐谷まつり</t>
+  </si>
+  <si>
+    <t>2019-11-23</t>
+  </si>
+  <si>
+    <t>ワンズファクトリー</t>
+  </si>
+  <si>
+    <t>WANZ</t>
+  </si>
+  <si>
+    <t>男潮吹きそのまま挿入、スプラッシュ中出し！</t>
+  </si>
+  <si>
+    <t>痴女、潮吹き、中出し、ハイビジョン、巨乳、単体作品、独占配信、手コキ</t>
+  </si>
+  <si>
+    <t>https://www.javbus.com/pics/cover/7f05_b.jpg</t>
+  </si>
+  <si>
     <t>假名</t>
   </si>
   <si>
@@ -285,6 +423,42 @@
     <t>label_000002</t>
   </si>
   <si>
+    <t>maker_000003</t>
+  </si>
+  <si>
+    <t>label_000003</t>
+  </si>
+  <si>
+    <t>https://www.javbus.com/pics/thumb/83ie.jpg</t>
+  </si>
+  <si>
+    <t>0</t>
+  </si>
+  <si>
+    <t>maker_000004</t>
+  </si>
+  <si>
+    <t>label_000004</t>
+  </si>
+  <si>
+    <t>https://www.javbus.com/pics/thumb/5klt.jpg</t>
+  </si>
+  <si>
+    <t>https://www.javbus.com/pics/thumb/649d.jpg</t>
+  </si>
+  <si>
+    <t>maker_000005</t>
+  </si>
+  <si>
+    <t>label_000005</t>
+  </si>
+  <si>
+    <t>series_000001</t>
+  </si>
+  <si>
+    <t>https://www.javbus.com/pics/thumb/7f05.jpg</t>
+  </si>
+  <si>
     <t>番号记录ID</t>
   </si>
   <si>
@@ -318,6 +492,42 @@
     <t>source_000004</t>
   </si>
   <si>
+    <t>code_000003</t>
+  </si>
+  <si>
+    <t>SSIS001</t>
+  </si>
+  <si>
+    <t>source_000005</t>
+  </si>
+  <si>
+    <t>code_000004</t>
+  </si>
+  <si>
+    <t>MIDE345</t>
+  </si>
+  <si>
+    <t>source_000006</t>
+  </si>
+  <si>
+    <t>code_000005</t>
+  </si>
+  <si>
+    <t>IPX001</t>
+  </si>
+  <si>
+    <t>source_000007</t>
+  </si>
+  <si>
+    <t>code_000006</t>
+  </si>
+  <si>
+    <t>WANZ912</t>
+  </si>
+  <si>
+    <t>source_000008</t>
+  </si>
+  <si>
     <t>角色/身份</t>
   </si>
   <si>
@@ -351,12 +561,81 @@
     <t>genre_000007</t>
   </si>
   <si>
+    <t>genre_000008</t>
+  </si>
+  <si>
+    <t>genre_000009</t>
+  </si>
+  <si>
+    <t>genre_000010</t>
+  </si>
+  <si>
+    <t>genre_000011</t>
+  </si>
+  <si>
+    <t>genre_000012</t>
+  </si>
+  <si>
+    <t>genre_000013</t>
+  </si>
+  <si>
+    <t>genre_000014</t>
+  </si>
+  <si>
+    <t>genre_000015</t>
+  </si>
+  <si>
+    <t>genre_000016</t>
+  </si>
+  <si>
+    <t>genre_000017</t>
+  </si>
+  <si>
+    <t>genre_000018</t>
+  </si>
+  <si>
+    <t>genre_000019</t>
+  </si>
+  <si>
+    <t>genre_000020</t>
+  </si>
+  <si>
+    <t>genre_000021</t>
+  </si>
+  <si>
+    <t>genre_000022</t>
+  </si>
+  <si>
+    <t>genre_000023</t>
+  </si>
+  <si>
+    <t>genre_000024</t>
+  </si>
+  <si>
+    <t>genre_000025</t>
+  </si>
+  <si>
+    <t>genre_000026</t>
+  </si>
+  <si>
+    <t>genre_000027</t>
+  </si>
+  <si>
     <t>导演ID</t>
   </si>
   <si>
     <t>director_000001</t>
   </si>
   <si>
+    <t>director_000002</t>
+  </si>
+  <si>
+    <t>director_000003</t>
+  </si>
+  <si>
+    <t>director_000004</t>
+  </si>
+  <si>
     <t>名称</t>
   </si>
   <si>
@@ -411,6 +690,126 @@
     <t>slender</t>
   </si>
   <si>
+    <t>3P・4P</t>
+  </si>
+  <si>
+    <t>metatube-JavBus-3200468f1f</t>
+  </si>
+  <si>
+    <t>美乳</t>
+  </si>
+  <si>
+    <t>metatube-JavBus-4464f10587</t>
+  </si>
+  <si>
+    <t>ギリモザ</t>
+  </si>
+  <si>
+    <t>metatube-JavBus-f2fa31e270</t>
+  </si>
+  <si>
+    <t>ハイビジョン</t>
+  </si>
+  <si>
+    <t>metatube-JavBus-6a63da99f0</t>
+  </si>
+  <si>
+    <t>寝取り・寝取られ</t>
+  </si>
+  <si>
+    <t>metatube-JavBus-7017909de1</t>
+  </si>
+  <si>
+    <t>ドラマ</t>
+  </si>
+  <si>
+    <t>metatube-JavBus-77bf3dd73e</t>
+  </si>
+  <si>
+    <t>独占配信</t>
+  </si>
+  <si>
+    <t>metatube-JavBus-772cdec556</t>
+  </si>
+  <si>
+    <t>淫語</t>
+  </si>
+  <si>
+    <t>metatube-JavBus-8d3154b878</t>
+  </si>
+  <si>
+    <t>デジモ</t>
+  </si>
+  <si>
+    <t>metatube-JavBus-c39811b970</t>
+  </si>
+  <si>
+    <t>主観</t>
+  </si>
+  <si>
+    <t>metatube-JavBus-e55126756e</t>
+  </si>
+  <si>
+    <t>顔面騎乗</t>
+  </si>
+  <si>
+    <t>metatube-JavBus-8cdb2c7dc0</t>
+  </si>
+  <si>
+    <t>巨乳</t>
+  </si>
+  <si>
+    <t>metatube-JavBus-f7f4f3529b</t>
+  </si>
+  <si>
+    <t>単体作品</t>
+  </si>
+  <si>
+    <t>metatube-JavBus-2d5a1de18a</t>
+  </si>
+  <si>
+    <t>ハメ撮り</t>
+  </si>
+  <si>
+    <t>metatube-JavBus-b03ff91d92</t>
+  </si>
+  <si>
+    <t>イラマチオ</t>
+  </si>
+  <si>
+    <t>metatube-JavBus-426b690eb8</t>
+  </si>
+  <si>
+    <t>女子校生</t>
+  </si>
+  <si>
+    <t>metatube-JavBus-370256efd8</t>
+  </si>
+  <si>
+    <t>痴女</t>
+  </si>
+  <si>
+    <t>metatube-JavBus-42b6825023</t>
+  </si>
+  <si>
+    <t>潮吹き</t>
+  </si>
+  <si>
+    <t>metatube-JavBus-9cdef30322</t>
+  </si>
+  <si>
+    <t>中出し</t>
+  </si>
+  <si>
+    <t>metatube-JavBus-3fe20114f3</t>
+  </si>
+  <si>
+    <t>手コキ</t>
+  </si>
+  <si>
+    <t>metatube-JavBus-ccb8c72421</t>
+  </si>
+  <si>
     <t>实体类型</t>
   </si>
   <si>
@@ -487,6 +886,60 @@
   </si>
   <si>
     <t>c6eea09a0ca201e4de5842fd46f2add11f3a8a11e7af794492da1c69c784fc08</t>
+  </si>
+  <si>
+    <t>metatube-bulk</t>
+  </si>
+  <si>
+    <t>JavBus:SSIS-001</t>
+  </si>
+  <si>
+    <t>https://www.javbus.com/ja/SSIS-001</t>
+  </si>
+  <si>
+    <t>2026-09-04T08:56:34.680Z</t>
+  </si>
+  <si>
+    <t>649f763a9c840d75e57b0354ad115a2378cd3b8bf31d8ddd6b3dabf340fae324</t>
+  </si>
+  <si>
+    <t>通过 MetaTube server 获取；上游 provider=JavBus；MetaTube 聚合多源，本记录仅代表 JavBus 一家；日文源</t>
+  </si>
+  <si>
+    <t>JavBus:MIDE-345</t>
+  </si>
+  <si>
+    <t>https://www.javbus.com/ja/MIDE-345</t>
+  </si>
+  <si>
+    <t>2026-09-04T08:56:36.689Z</t>
+  </si>
+  <si>
+    <t>eccdb0254fc2dc9f9233374d1dbbda1040131512909cad9a4ef2249c1d41ec7b</t>
+  </si>
+  <si>
+    <t>JavBus:IPX-001</t>
+  </si>
+  <si>
+    <t>https://www.javbus.com/ja/IPX-001</t>
+  </si>
+  <si>
+    <t>2026-09-04T08:56:38.702Z</t>
+  </si>
+  <si>
+    <t>eea891d314431d5bf7d885593d966a380b273920451f2055aa5d08cfc8e0dca7</t>
+  </si>
+  <si>
+    <t>JavBus:WANZ-912</t>
+  </si>
+  <si>
+    <t>https://www.javbus.com/ja/WANZ-912</t>
+  </si>
+  <si>
+    <t>2026-09-04T08:56:40.712Z</t>
+  </si>
+  <si>
+    <t>f72c0ba9de8b34a573d01afe61328ec72130c5ca56af151074fe426e1c0aa146</t>
   </si>
 </sst>
 </file>
@@ -891,7 +1344,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:R3"/>
+  <dimension ref="A1:R8"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="18" customWidth="1"/>
@@ -1072,8 +1525,278 @@
         <v>30</v>
       </c>
     </row>
+    <row r="4" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="A4" s="3" t="s">
+        <v>31</v>
+      </c>
+      <c r="B4" s="3" t="s">
+        <v>32</v>
+      </c>
+      <c r="C4" s="3" t="s">
+        <v>32</v>
+      </c>
+      <c r="D4" s="3" t="s">
+        <v>22</v>
+      </c>
+      <c r="E4" s="3" t="s">
+        <v>22</v>
+      </c>
+      <c r="F4" s="3" t="s">
+        <v>21</v>
+      </c>
+      <c r="G4" s="3" t="s">
+        <v>22</v>
+      </c>
+      <c r="H4" s="3" t="s">
+        <v>22</v>
+      </c>
+      <c r="I4" s="3" t="s">
+        <v>22</v>
+      </c>
+      <c r="J4" s="3"/>
+      <c r="K4" s="3" t="s">
+        <v>22</v>
+      </c>
+      <c r="L4" s="3" t="s">
+        <v>22</v>
+      </c>
+      <c r="M4" s="3" t="s">
+        <v>22</v>
+      </c>
+      <c r="N4" s="3" t="s">
+        <v>22</v>
+      </c>
+      <c r="O4" s="3">
+        <v>1</v>
+      </c>
+      <c r="P4" s="3" t="s">
+        <v>22</v>
+      </c>
+      <c r="Q4" s="3" t="s">
+        <v>22</v>
+      </c>
+      <c r="R4" s="3" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="5" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="A5" s="3" t="s">
+        <v>34</v>
+      </c>
+      <c r="B5" s="3" t="s">
+        <v>35</v>
+      </c>
+      <c r="C5" s="3" t="s">
+        <v>35</v>
+      </c>
+      <c r="D5" s="3" t="s">
+        <v>22</v>
+      </c>
+      <c r="E5" s="3" t="s">
+        <v>22</v>
+      </c>
+      <c r="F5" s="3" t="s">
+        <v>21</v>
+      </c>
+      <c r="G5" s="3" t="s">
+        <v>22</v>
+      </c>
+      <c r="H5" s="3" t="s">
+        <v>22</v>
+      </c>
+      <c r="I5" s="3" t="s">
+        <v>22</v>
+      </c>
+      <c r="J5" s="3"/>
+      <c r="K5" s="3" t="s">
+        <v>22</v>
+      </c>
+      <c r="L5" s="3" t="s">
+        <v>22</v>
+      </c>
+      <c r="M5" s="3" t="s">
+        <v>22</v>
+      </c>
+      <c r="N5" s="3" t="s">
+        <v>22</v>
+      </c>
+      <c r="O5" s="3">
+        <v>1</v>
+      </c>
+      <c r="P5" s="3" t="s">
+        <v>22</v>
+      </c>
+      <c r="Q5" s="3" t="s">
+        <v>22</v>
+      </c>
+      <c r="R5" s="3" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="6" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="A6" s="3" t="s">
+        <v>36</v>
+      </c>
+      <c r="B6" s="3" t="s">
+        <v>37</v>
+      </c>
+      <c r="C6" s="3" t="s">
+        <v>22</v>
+      </c>
+      <c r="D6" s="3" t="s">
+        <v>37</v>
+      </c>
+      <c r="E6" s="3" t="s">
+        <v>22</v>
+      </c>
+      <c r="F6" s="3" t="s">
+        <v>21</v>
+      </c>
+      <c r="G6" s="3" t="s">
+        <v>22</v>
+      </c>
+      <c r="H6" s="3" t="s">
+        <v>22</v>
+      </c>
+      <c r="I6" s="3" t="s">
+        <v>22</v>
+      </c>
+      <c r="J6" s="3"/>
+      <c r="K6" s="3" t="s">
+        <v>22</v>
+      </c>
+      <c r="L6" s="3" t="s">
+        <v>22</v>
+      </c>
+      <c r="M6" s="3" t="s">
+        <v>22</v>
+      </c>
+      <c r="N6" s="3" t="s">
+        <v>22</v>
+      </c>
+      <c r="O6" s="3">
+        <v>1</v>
+      </c>
+      <c r="P6" s="3" t="s">
+        <v>22</v>
+      </c>
+      <c r="Q6" s="3" t="s">
+        <v>22</v>
+      </c>
+      <c r="R6" s="3" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="7" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="A7" s="3" t="s">
+        <v>38</v>
+      </c>
+      <c r="B7" s="3" t="s">
+        <v>39</v>
+      </c>
+      <c r="C7" s="3" t="s">
+        <v>39</v>
+      </c>
+      <c r="D7" s="3" t="s">
+        <v>22</v>
+      </c>
+      <c r="E7" s="3" t="s">
+        <v>22</v>
+      </c>
+      <c r="F7" s="3" t="s">
+        <v>21</v>
+      </c>
+      <c r="G7" s="3" t="s">
+        <v>22</v>
+      </c>
+      <c r="H7" s="3" t="s">
+        <v>22</v>
+      </c>
+      <c r="I7" s="3" t="s">
+        <v>22</v>
+      </c>
+      <c r="J7" s="3"/>
+      <c r="K7" s="3" t="s">
+        <v>22</v>
+      </c>
+      <c r="L7" s="3" t="s">
+        <v>22</v>
+      </c>
+      <c r="M7" s="3" t="s">
+        <v>22</v>
+      </c>
+      <c r="N7" s="3" t="s">
+        <v>22</v>
+      </c>
+      <c r="O7" s="3">
+        <v>1</v>
+      </c>
+      <c r="P7" s="3" t="s">
+        <v>22</v>
+      </c>
+      <c r="Q7" s="3" t="s">
+        <v>22</v>
+      </c>
+      <c r="R7" s="3" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="8" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="A8" s="3" t="s">
+        <v>40</v>
+      </c>
+      <c r="B8" s="3" t="s">
+        <v>41</v>
+      </c>
+      <c r="C8" s="3" t="s">
+        <v>41</v>
+      </c>
+      <c r="D8" s="3" t="s">
+        <v>22</v>
+      </c>
+      <c r="E8" s="3" t="s">
+        <v>22</v>
+      </c>
+      <c r="F8" s="3" t="s">
+        <v>21</v>
+      </c>
+      <c r="G8" s="3" t="s">
+        <v>22</v>
+      </c>
+      <c r="H8" s="3" t="s">
+        <v>22</v>
+      </c>
+      <c r="I8" s="3" t="s">
+        <v>22</v>
+      </c>
+      <c r="J8" s="3"/>
+      <c r="K8" s="3" t="s">
+        <v>22</v>
+      </c>
+      <c r="L8" s="3" t="s">
+        <v>22</v>
+      </c>
+      <c r="M8" s="3" t="s">
+        <v>22</v>
+      </c>
+      <c r="N8" s="3" t="s">
+        <v>22</v>
+      </c>
+      <c r="O8" s="3">
+        <v>1</v>
+      </c>
+      <c r="P8" s="3" t="s">
+        <v>22</v>
+      </c>
+      <c r="Q8" s="3" t="s">
+        <v>22</v>
+      </c>
+      <c r="R8" s="3" t="s">
+        <v>33</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:R3"/>
+  <autoFilter ref="A1:R8"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
 </worksheet>
@@ -1081,12 +1804,11 @@
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:G3"/>
+  <dimension ref="A1:G6"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="16" customWidth="1"/>
-    <col min="2" max="2" width="15" customWidth="1"/>
-    <col min="3" max="3" width="12" customWidth="1"/>
+    <col min="2" max="3" width="19" customWidth="1"/>
     <col min="4" max="4" width="23" customWidth="1"/>
     <col min="5" max="5" width="12" customWidth="1"/>
     <col min="6" max="7" width="24" customWidth="1"/>
@@ -1094,22 +1816,22 @@
   <sheetData>
     <row r="1" ht="24" customHeight="1" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="5" t="s">
-        <v>75</v>
+        <v>121</v>
       </c>
       <c r="B1" s="5" t="s">
-        <v>110</v>
+        <v>203</v>
       </c>
       <c r="C1" s="5" t="s">
         <v>2</v>
       </c>
       <c r="D1" s="5" t="s">
-        <v>111</v>
+        <v>204</v>
       </c>
       <c r="E1" s="5" t="s">
         <v>16</v>
       </c>
       <c r="F1" s="5" t="s">
-        <v>63</v>
+        <v>109</v>
       </c>
       <c r="G1" s="5" t="s">
         <v>17</v>
@@ -1117,16 +1839,16 @@
     </row>
     <row r="2" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A2" s="3" t="s">
-        <v>81</v>
+        <v>127</v>
       </c>
       <c r="B2" s="3" t="s">
-        <v>47</v>
+        <v>58</v>
       </c>
       <c r="C2" s="3" t="s">
-        <v>47</v>
+        <v>58</v>
       </c>
       <c r="D2" s="3" t="s">
-        <v>112</v>
+        <v>205</v>
       </c>
       <c r="E2" s="3"/>
       <c r="F2" s="3" t="s">
@@ -1138,10 +1860,10 @@
     </row>
     <row r="3" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A3" s="3" t="s">
-        <v>84</v>
+        <v>130</v>
       </c>
       <c r="B3" s="3" t="s">
-        <v>56</v>
+        <v>67</v>
       </c>
       <c r="C3" s="3"/>
       <c r="D3" s="3"/>
@@ -1153,8 +1875,65 @@
         <v>30</v>
       </c>
     </row>
+    <row r="4" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A4" s="3" t="s">
+        <v>132</v>
+      </c>
+      <c r="B4" s="3" t="s">
+        <v>75</v>
+      </c>
+      <c r="C4" s="3" t="s">
+        <v>75</v>
+      </c>
+      <c r="D4" s="3"/>
+      <c r="E4" s="3"/>
+      <c r="F4" s="3" t="s">
+        <v>33</v>
+      </c>
+      <c r="G4" s="3" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="5" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A5" s="3" t="s">
+        <v>136</v>
+      </c>
+      <c r="B5" s="3" t="s">
+        <v>84</v>
+      </c>
+      <c r="C5" s="3" t="s">
+        <v>84</v>
+      </c>
+      <c r="D5" s="3"/>
+      <c r="E5" s="3"/>
+      <c r="F5" s="3" t="s">
+        <v>33</v>
+      </c>
+      <c r="G5" s="3" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="6" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A6" s="3" t="s">
+        <v>140</v>
+      </c>
+      <c r="B6" s="3" t="s">
+        <v>100</v>
+      </c>
+      <c r="C6" s="3" t="s">
+        <v>100</v>
+      </c>
+      <c r="D6" s="3"/>
+      <c r="E6" s="3"/>
+      <c r="F6" s="3" t="s">
+        <v>33</v>
+      </c>
+      <c r="G6" s="3" t="s">
+        <v>33</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:G3"/>
+  <autoFilter ref="A1:G6"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
 </worksheet>
@@ -1162,36 +1941,37 @@
 
 <file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:H3"/>
+  <dimension ref="A1:H6"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="2" width="16" customWidth="1"/>
-    <col min="3" max="4" width="13" customWidth="1"/>
+    <col min="3" max="3" width="17" customWidth="1"/>
+    <col min="4" max="4" width="13" customWidth="1"/>
     <col min="5" max="6" width="12" customWidth="1"/>
     <col min="7" max="8" width="24" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" ht="24" customHeight="1" spans="1:8" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="5" t="s">
-        <v>76</v>
+        <v>122</v>
       </c>
       <c r="B1" s="5" t="s">
-        <v>75</v>
+        <v>121</v>
       </c>
       <c r="C1" s="5" t="s">
-        <v>110</v>
+        <v>203</v>
       </c>
       <c r="D1" s="5" t="s">
         <v>2</v>
       </c>
       <c r="E1" s="5" t="s">
-        <v>111</v>
+        <v>204</v>
       </c>
       <c r="F1" s="5" t="s">
         <v>16</v>
       </c>
       <c r="G1" s="5" t="s">
-        <v>63</v>
+        <v>109</v>
       </c>
       <c r="H1" s="5" t="s">
         <v>17</v>
@@ -1199,16 +1979,16 @@
     </row>
     <row r="2" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A2" s="3" t="s">
-        <v>82</v>
+        <v>128</v>
       </c>
       <c r="B2" s="3" t="s">
-        <v>81</v>
+        <v>127</v>
       </c>
       <c r="C2" s="3" t="s">
-        <v>48</v>
+        <v>59</v>
       </c>
       <c r="D2" s="3" t="s">
-        <v>48</v>
+        <v>59</v>
       </c>
       <c r="E2" s="3"/>
       <c r="F2" s="3"/>
@@ -1221,13 +2001,13 @@
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A3" s="3" t="s">
-        <v>85</v>
+        <v>131</v>
       </c>
       <c r="B3" s="3" t="s">
-        <v>84</v>
+        <v>130</v>
       </c>
       <c r="C3" s="3" t="s">
-        <v>57</v>
+        <v>68</v>
       </c>
       <c r="D3" s="3"/>
       <c r="E3" s="3"/>
@@ -1239,8 +2019,68 @@
         <v>30</v>
       </c>
     </row>
+    <row r="4" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A4" s="3" t="s">
+        <v>133</v>
+      </c>
+      <c r="B4" s="3" t="s">
+        <v>132</v>
+      </c>
+      <c r="C4" s="3" t="s">
+        <v>76</v>
+      </c>
+      <c r="D4" s="3"/>
+      <c r="E4" s="3"/>
+      <c r="F4" s="3"/>
+      <c r="G4" s="3" t="s">
+        <v>33</v>
+      </c>
+      <c r="H4" s="3" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="5" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A5" s="3" t="s">
+        <v>137</v>
+      </c>
+      <c r="B5" s="3" t="s">
+        <v>136</v>
+      </c>
+      <c r="C5" s="3" t="s">
+        <v>85</v>
+      </c>
+      <c r="D5" s="3"/>
+      <c r="E5" s="3"/>
+      <c r="F5" s="3"/>
+      <c r="G5" s="3" t="s">
+        <v>33</v>
+      </c>
+      <c r="H5" s="3" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="6" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A6" s="3" t="s">
+        <v>141</v>
+      </c>
+      <c r="B6" s="3" t="s">
+        <v>140</v>
+      </c>
+      <c r="C6" s="3" t="s">
+        <v>101</v>
+      </c>
+      <c r="D6" s="3"/>
+      <c r="E6" s="3"/>
+      <c r="F6" s="3"/>
+      <c r="G6" s="3" t="s">
+        <v>33</v>
+      </c>
+      <c r="H6" s="3" t="s">
+        <v>33</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:H3"/>
+  <autoFilter ref="A1:H6"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
 </worksheet>
@@ -1248,24 +2088,28 @@
 
 <file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:H1"/>
+  <dimension ref="A1:H2"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
-    <col min="1" max="8" width="12" customWidth="1"/>
+    <col min="1" max="1" width="17" customWidth="1"/>
+    <col min="2" max="3" width="16" customWidth="1"/>
+    <col min="4" max="5" width="25" customWidth="1"/>
+    <col min="6" max="6" width="12" customWidth="1"/>
+    <col min="7" max="8" width="24" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" ht="24" customHeight="1" spans="1:8" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="5" t="s">
-        <v>77</v>
+        <v>123</v>
       </c>
       <c r="B1" s="5" t="s">
-        <v>75</v>
+        <v>121</v>
       </c>
       <c r="C1" s="5" t="s">
-        <v>76</v>
+        <v>122</v>
       </c>
       <c r="D1" s="5" t="s">
-        <v>110</v>
+        <v>203</v>
       </c>
       <c r="E1" s="5" t="s">
         <v>2</v>
@@ -1274,14 +2118,38 @@
         <v>16</v>
       </c>
       <c r="G1" s="5" t="s">
-        <v>63</v>
+        <v>109</v>
       </c>
       <c r="H1" s="5" t="s">
         <v>17</v>
       </c>
     </row>
+    <row r="2" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A2" s="3" t="s">
+        <v>142</v>
+      </c>
+      <c r="B2" s="3" t="s">
+        <v>140</v>
+      </c>
+      <c r="C2" s="3" t="s">
+        <v>141</v>
+      </c>
+      <c r="D2" s="3" t="s">
+        <v>102</v>
+      </c>
+      <c r="E2" s="3" t="s">
+        <v>102</v>
+      </c>
+      <c r="F2" s="3"/>
+      <c r="G2" s="3" t="s">
+        <v>33</v>
+      </c>
+      <c r="H2" s="3" t="s">
+        <v>33</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:H1"/>
+  <autoFilter ref="A1:H2"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
 </worksheet>
@@ -1289,34 +2157,34 @@
 
 <file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:G8"/>
+  <dimension ref="A1:G28"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="16" customWidth="1"/>
     <col min="2" max="3" width="12" customWidth="1"/>
-    <col min="4" max="4" width="15" customWidth="1"/>
+    <col min="4" max="4" width="30" customWidth="1"/>
     <col min="5" max="5" width="12" customWidth="1"/>
     <col min="6" max="7" width="24" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" ht="24" customHeight="1" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="5" t="s">
-        <v>100</v>
+        <v>170</v>
       </c>
       <c r="B1" s="5" t="s">
-        <v>110</v>
+        <v>203</v>
       </c>
       <c r="C1" s="5" t="s">
         <v>2</v>
       </c>
       <c r="D1" s="5" t="s">
-        <v>113</v>
+        <v>206</v>
       </c>
       <c r="E1" s="5" t="s">
-        <v>114</v>
+        <v>207</v>
       </c>
       <c r="F1" s="5" t="s">
-        <v>63</v>
+        <v>109</v>
       </c>
       <c r="G1" s="5" t="s">
         <v>17</v>
@@ -1324,16 +2192,16 @@
     </row>
     <row r="2" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A2" s="3" t="s">
-        <v>101</v>
+        <v>171</v>
       </c>
       <c r="B2" s="3" t="s">
-        <v>115</v>
+        <v>208</v>
       </c>
       <c r="C2" s="3" t="s">
-        <v>115</v>
+        <v>208</v>
       </c>
       <c r="D2" s="3" t="s">
-        <v>116</v>
+        <v>209</v>
       </c>
       <c r="E2" s="3"/>
       <c r="F2" s="3" t="s">
@@ -1345,16 +2213,16 @@
     </row>
     <row r="3" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A3" s="3" t="s">
-        <v>102</v>
+        <v>172</v>
       </c>
       <c r="B3" s="3" t="s">
-        <v>117</v>
+        <v>210</v>
       </c>
       <c r="C3" s="3" t="s">
-        <v>117</v>
+        <v>210</v>
       </c>
       <c r="D3" s="3" t="s">
-        <v>118</v>
+        <v>211</v>
       </c>
       <c r="E3" s="3"/>
       <c r="F3" s="3" t="s">
@@ -1366,16 +2234,16 @@
     </row>
     <row r="4" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A4" s="3" t="s">
-        <v>103</v>
+        <v>173</v>
       </c>
       <c r="B4" s="3" t="s">
-        <v>119</v>
+        <v>212</v>
       </c>
       <c r="C4" s="3" t="s">
-        <v>119</v>
+        <v>212</v>
       </c>
       <c r="D4" s="3" t="s">
-        <v>120</v>
+        <v>213</v>
       </c>
       <c r="E4" s="3"/>
       <c r="F4" s="3" t="s">
@@ -1387,16 +2255,16 @@
     </row>
     <row r="5" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A5" s="3" t="s">
-        <v>104</v>
+        <v>174</v>
       </c>
       <c r="B5" s="3" t="s">
-        <v>121</v>
+        <v>214</v>
       </c>
       <c r="C5" s="3" t="s">
-        <v>121</v>
+        <v>214</v>
       </c>
       <c r="D5" s="3" t="s">
-        <v>122</v>
+        <v>215</v>
       </c>
       <c r="E5" s="3"/>
       <c r="F5" s="3" t="s">
@@ -1408,16 +2276,16 @@
     </row>
     <row r="6" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A6" s="3" t="s">
-        <v>105</v>
+        <v>175</v>
       </c>
       <c r="B6" s="3" t="s">
-        <v>123</v>
+        <v>216</v>
       </c>
       <c r="C6" s="3" t="s">
-        <v>123</v>
+        <v>216</v>
       </c>
       <c r="D6" s="3" t="s">
-        <v>124</v>
+        <v>217</v>
       </c>
       <c r="E6" s="3"/>
       <c r="F6" s="3" t="s">
@@ -1429,16 +2297,16 @@
     </row>
     <row r="7" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A7" s="3" t="s">
-        <v>106</v>
+        <v>176</v>
       </c>
       <c r="B7" s="3" t="s">
-        <v>125</v>
+        <v>218</v>
       </c>
       <c r="C7" s="3" t="s">
-        <v>125</v>
+        <v>218</v>
       </c>
       <c r="D7" s="3" t="s">
-        <v>126</v>
+        <v>219</v>
       </c>
       <c r="E7" s="3"/>
       <c r="F7" s="3" t="s">
@@ -1450,14 +2318,14 @@
     </row>
     <row r="8" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A8" s="3" t="s">
-        <v>107</v>
+        <v>177</v>
       </c>
       <c r="B8" s="3" t="s">
-        <v>58</v>
+        <v>69</v>
       </c>
       <c r="C8" s="3"/>
       <c r="D8" s="3" t="s">
-        <v>127</v>
+        <v>220</v>
       </c>
       <c r="E8" s="3"/>
       <c r="F8" s="3" t="s">
@@ -1467,8 +2335,428 @@
         <v>30</v>
       </c>
     </row>
+    <row r="9" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A9" s="3" t="s">
+        <v>178</v>
+      </c>
+      <c r="B9" s="3" t="s">
+        <v>221</v>
+      </c>
+      <c r="C9" s="3" t="s">
+        <v>221</v>
+      </c>
+      <c r="D9" s="3" t="s">
+        <v>222</v>
+      </c>
+      <c r="E9" s="3"/>
+      <c r="F9" s="3" t="s">
+        <v>33</v>
+      </c>
+      <c r="G9" s="3" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="10" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A10" s="3" t="s">
+        <v>179</v>
+      </c>
+      <c r="B10" s="3" t="s">
+        <v>223</v>
+      </c>
+      <c r="C10" s="3" t="s">
+        <v>223</v>
+      </c>
+      <c r="D10" s="3" t="s">
+        <v>224</v>
+      </c>
+      <c r="E10" s="3"/>
+      <c r="F10" s="3" t="s">
+        <v>33</v>
+      </c>
+      <c r="G10" s="3" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="11" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A11" s="3" t="s">
+        <v>180</v>
+      </c>
+      <c r="B11" s="3" t="s">
+        <v>225</v>
+      </c>
+      <c r="C11" s="3" t="s">
+        <v>225</v>
+      </c>
+      <c r="D11" s="3" t="s">
+        <v>226</v>
+      </c>
+      <c r="E11" s="3"/>
+      <c r="F11" s="3" t="s">
+        <v>33</v>
+      </c>
+      <c r="G11" s="3" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="12" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A12" s="3" t="s">
+        <v>181</v>
+      </c>
+      <c r="B12" s="3" t="s">
+        <v>227</v>
+      </c>
+      <c r="C12" s="3" t="s">
+        <v>227</v>
+      </c>
+      <c r="D12" s="3" t="s">
+        <v>228</v>
+      </c>
+      <c r="E12" s="3"/>
+      <c r="F12" s="3" t="s">
+        <v>33</v>
+      </c>
+      <c r="G12" s="3" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="13" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A13" s="3" t="s">
+        <v>182</v>
+      </c>
+      <c r="B13" s="3" t="s">
+        <v>229</v>
+      </c>
+      <c r="C13" s="3" t="s">
+        <v>229</v>
+      </c>
+      <c r="D13" s="3" t="s">
+        <v>230</v>
+      </c>
+      <c r="E13" s="3"/>
+      <c r="F13" s="3" t="s">
+        <v>33</v>
+      </c>
+      <c r="G13" s="3" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="14" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A14" s="3" t="s">
+        <v>183</v>
+      </c>
+      <c r="B14" s="3" t="s">
+        <v>231</v>
+      </c>
+      <c r="C14" s="3" t="s">
+        <v>231</v>
+      </c>
+      <c r="D14" s="3" t="s">
+        <v>232</v>
+      </c>
+      <c r="E14" s="3"/>
+      <c r="F14" s="3" t="s">
+        <v>33</v>
+      </c>
+      <c r="G14" s="3" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="15" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A15" s="3" t="s">
+        <v>184</v>
+      </c>
+      <c r="B15" s="3" t="s">
+        <v>233</v>
+      </c>
+      <c r="C15" s="3" t="s">
+        <v>233</v>
+      </c>
+      <c r="D15" s="3" t="s">
+        <v>234</v>
+      </c>
+      <c r="E15" s="3"/>
+      <c r="F15" s="3" t="s">
+        <v>33</v>
+      </c>
+      <c r="G15" s="3" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="16" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A16" s="3" t="s">
+        <v>185</v>
+      </c>
+      <c r="B16" s="3" t="s">
+        <v>235</v>
+      </c>
+      <c r="C16" s="3" t="s">
+        <v>235</v>
+      </c>
+      <c r="D16" s="3" t="s">
+        <v>236</v>
+      </c>
+      <c r="E16" s="3"/>
+      <c r="F16" s="3" t="s">
+        <v>33</v>
+      </c>
+      <c r="G16" s="3" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="17" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A17" s="3" t="s">
+        <v>186</v>
+      </c>
+      <c r="B17" s="3" t="s">
+        <v>237</v>
+      </c>
+      <c r="C17" s="3" t="s">
+        <v>237</v>
+      </c>
+      <c r="D17" s="3" t="s">
+        <v>238</v>
+      </c>
+      <c r="E17" s="3"/>
+      <c r="F17" s="3" t="s">
+        <v>33</v>
+      </c>
+      <c r="G17" s="3" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="18" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A18" s="3" t="s">
+        <v>187</v>
+      </c>
+      <c r="B18" s="3" t="s">
+        <v>239</v>
+      </c>
+      <c r="C18" s="3" t="s">
+        <v>239</v>
+      </c>
+      <c r="D18" s="3" t="s">
+        <v>240</v>
+      </c>
+      <c r="E18" s="3"/>
+      <c r="F18" s="3" t="s">
+        <v>33</v>
+      </c>
+      <c r="G18" s="3" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="19" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A19" s="3" t="s">
+        <v>188</v>
+      </c>
+      <c r="B19" s="3" t="s">
+        <v>241</v>
+      </c>
+      <c r="C19" s="3" t="s">
+        <v>241</v>
+      </c>
+      <c r="D19" s="3" t="s">
+        <v>242</v>
+      </c>
+      <c r="E19" s="3"/>
+      <c r="F19" s="3" t="s">
+        <v>33</v>
+      </c>
+      <c r="G19" s="3" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="20" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A20" s="3" t="s">
+        <v>189</v>
+      </c>
+      <c r="B20" s="3" t="s">
+        <v>243</v>
+      </c>
+      <c r="C20" s="3" t="s">
+        <v>243</v>
+      </c>
+      <c r="D20" s="3" t="s">
+        <v>244</v>
+      </c>
+      <c r="E20" s="3"/>
+      <c r="F20" s="3" t="s">
+        <v>33</v>
+      </c>
+      <c r="G20" s="3" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="21" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A21" s="3" t="s">
+        <v>190</v>
+      </c>
+      <c r="B21" s="3" t="s">
+        <v>245</v>
+      </c>
+      <c r="C21" s="3" t="s">
+        <v>245</v>
+      </c>
+      <c r="D21" s="3" t="s">
+        <v>246</v>
+      </c>
+      <c r="E21" s="3"/>
+      <c r="F21" s="3" t="s">
+        <v>33</v>
+      </c>
+      <c r="G21" s="3" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="22" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A22" s="3" t="s">
+        <v>191</v>
+      </c>
+      <c r="B22" s="3" t="s">
+        <v>247</v>
+      </c>
+      <c r="C22" s="3" t="s">
+        <v>247</v>
+      </c>
+      <c r="D22" s="3" t="s">
+        <v>248</v>
+      </c>
+      <c r="E22" s="3"/>
+      <c r="F22" s="3" t="s">
+        <v>33</v>
+      </c>
+      <c r="G22" s="3" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="23" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A23" s="3" t="s">
+        <v>192</v>
+      </c>
+      <c r="B23" s="3" t="s">
+        <v>249</v>
+      </c>
+      <c r="C23" s="3" t="s">
+        <v>249</v>
+      </c>
+      <c r="D23" s="3" t="s">
+        <v>250</v>
+      </c>
+      <c r="E23" s="3"/>
+      <c r="F23" s="3" t="s">
+        <v>33</v>
+      </c>
+      <c r="G23" s="3" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="24" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A24" s="3" t="s">
+        <v>193</v>
+      </c>
+      <c r="B24" s="3" t="s">
+        <v>251</v>
+      </c>
+      <c r="C24" s="3" t="s">
+        <v>251</v>
+      </c>
+      <c r="D24" s="3" t="s">
+        <v>252</v>
+      </c>
+      <c r="E24" s="3"/>
+      <c r="F24" s="3" t="s">
+        <v>33</v>
+      </c>
+      <c r="G24" s="3" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="25" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A25" s="3" t="s">
+        <v>194</v>
+      </c>
+      <c r="B25" s="3" t="s">
+        <v>253</v>
+      </c>
+      <c r="C25" s="3" t="s">
+        <v>253</v>
+      </c>
+      <c r="D25" s="3" t="s">
+        <v>254</v>
+      </c>
+      <c r="E25" s="3"/>
+      <c r="F25" s="3" t="s">
+        <v>33</v>
+      </c>
+      <c r="G25" s="3" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="26" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A26" s="3" t="s">
+        <v>195</v>
+      </c>
+      <c r="B26" s="3" t="s">
+        <v>255</v>
+      </c>
+      <c r="C26" s="3" t="s">
+        <v>255</v>
+      </c>
+      <c r="D26" s="3" t="s">
+        <v>256</v>
+      </c>
+      <c r="E26" s="3"/>
+      <c r="F26" s="3" t="s">
+        <v>33</v>
+      </c>
+      <c r="G26" s="3" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="27" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A27" s="3" t="s">
+        <v>196</v>
+      </c>
+      <c r="B27" s="3" t="s">
+        <v>257</v>
+      </c>
+      <c r="C27" s="3" t="s">
+        <v>257</v>
+      </c>
+      <c r="D27" s="3" t="s">
+        <v>258</v>
+      </c>
+      <c r="E27" s="3"/>
+      <c r="F27" s="3" t="s">
+        <v>33</v>
+      </c>
+      <c r="G27" s="3" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="28" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A28" s="3" t="s">
+        <v>197</v>
+      </c>
+      <c r="B28" s="3" t="s">
+        <v>259</v>
+      </c>
+      <c r="C28" s="3" t="s">
+        <v>259</v>
+      </c>
+      <c r="D28" s="3" t="s">
+        <v>260</v>
+      </c>
+      <c r="E28" s="3"/>
+      <c r="F28" s="3" t="s">
+        <v>33</v>
+      </c>
+      <c r="G28" s="3" t="s">
+        <v>33</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:G8"/>
+  <autoFilter ref="A1:G28"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
 </worksheet>
@@ -1476,7 +2764,7 @@
 
 <file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:G2"/>
+  <dimension ref="A1:G5"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="19" customWidth="1"/>
@@ -1486,22 +2774,22 @@
   <sheetData>
     <row r="1" ht="24" customHeight="1" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="5" t="s">
-        <v>108</v>
+        <v>198</v>
       </c>
       <c r="B1" s="5" t="s">
-        <v>110</v>
+        <v>203</v>
       </c>
       <c r="C1" s="5" t="s">
         <v>2</v>
       </c>
       <c r="D1" s="5" t="s">
-        <v>111</v>
+        <v>204</v>
       </c>
       <c r="E1" s="5" t="s">
         <v>16</v>
       </c>
       <c r="F1" s="5" t="s">
-        <v>63</v>
+        <v>109</v>
       </c>
       <c r="G1" s="5" t="s">
         <v>17</v>
@@ -1509,13 +2797,13 @@
     </row>
     <row r="2" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A2" s="3" t="s">
-        <v>109</v>
+        <v>199</v>
       </c>
       <c r="B2" s="3" t="s">
-        <v>49</v>
+        <v>60</v>
       </c>
       <c r="C2" s="3" t="s">
-        <v>49</v>
+        <v>60</v>
       </c>
       <c r="D2" s="3"/>
       <c r="E2" s="3"/>
@@ -1526,8 +2814,65 @@
         <v>26</v>
       </c>
     </row>
+    <row r="3" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A3" s="3" t="s">
+        <v>200</v>
+      </c>
+      <c r="B3" s="3" t="s">
+        <v>77</v>
+      </c>
+      <c r="C3" s="3" t="s">
+        <v>77</v>
+      </c>
+      <c r="D3" s="3"/>
+      <c r="E3" s="3"/>
+      <c r="F3" s="3" t="s">
+        <v>33</v>
+      </c>
+      <c r="G3" s="3" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="4" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A4" s="3" t="s">
+        <v>201</v>
+      </c>
+      <c r="B4" s="3" t="s">
+        <v>86</v>
+      </c>
+      <c r="C4" s="3" t="s">
+        <v>86</v>
+      </c>
+      <c r="D4" s="3"/>
+      <c r="E4" s="3"/>
+      <c r="F4" s="3" t="s">
+        <v>33</v>
+      </c>
+      <c r="G4" s="3" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="5" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A5" s="3" t="s">
+        <v>202</v>
+      </c>
+      <c r="B5" s="3" t="s">
+        <v>93</v>
+      </c>
+      <c r="C5" s="3" t="s">
+        <v>93</v>
+      </c>
+      <c r="D5" s="3"/>
+      <c r="E5" s="3"/>
+      <c r="F5" s="3" t="s">
+        <v>33</v>
+      </c>
+      <c r="G5" s="3" t="s">
+        <v>33</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:G2"/>
+  <autoFilter ref="A1:G5"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
 </worksheet>
@@ -1535,7 +2880,7 @@
 
 <file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:I5"/>
+  <dimension ref="A1:I9"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="17" customWidth="1"/>
@@ -1545,145 +2890,260 @@
     <col min="5" max="5" width="27" customWidth="1"/>
     <col min="6" max="6" width="40" customWidth="1"/>
     <col min="7" max="7" width="28" customWidth="1"/>
-    <col min="8" max="8" width="40" customWidth="1"/>
-    <col min="9" max="9" width="12" customWidth="1"/>
+    <col min="8" max="9" width="40" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" ht="24" customHeight="1" spans="1:9" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="5" t="s">
-        <v>69</v>
+        <v>115</v>
       </c>
       <c r="B1" s="5" t="s">
-        <v>128</v>
+        <v>261</v>
       </c>
       <c r="C1" s="5" t="s">
-        <v>129</v>
+        <v>262</v>
       </c>
       <c r="D1" s="5" t="s">
-        <v>130</v>
+        <v>263</v>
       </c>
       <c r="E1" s="5" t="s">
-        <v>131</v>
+        <v>264</v>
       </c>
       <c r="F1" s="5" t="s">
-        <v>132</v>
+        <v>265</v>
       </c>
       <c r="G1" s="5" t="s">
-        <v>133</v>
+        <v>266</v>
       </c>
       <c r="H1" s="5" t="s">
-        <v>134</v>
+        <v>267</v>
       </c>
       <c r="I1" s="5" t="s">
-        <v>135</v>
+        <v>268</v>
       </c>
     </row>
     <row r="2" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A2" s="3" t="s">
-        <v>136</v>
+        <v>269</v>
       </c>
       <c r="B2" s="3" t="s">
-        <v>99</v>
+        <v>169</v>
       </c>
       <c r="C2" s="3" t="s">
         <v>18</v>
       </c>
       <c r="D2" s="3" t="s">
-        <v>137</v>
+        <v>270</v>
       </c>
       <c r="E2" s="3" t="s">
-        <v>138</v>
+        <v>271</v>
       </c>
       <c r="F2" s="3" t="s">
-        <v>139</v>
+        <v>272</v>
       </c>
       <c r="G2" s="3" t="s">
-        <v>140</v>
+        <v>273</v>
       </c>
       <c r="H2" s="3" t="s">
-        <v>141</v>
+        <v>274</v>
       </c>
       <c r="I2" s="3"/>
     </row>
     <row r="3" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A3" s="3" t="s">
-        <v>93</v>
+        <v>151</v>
       </c>
       <c r="B3" s="3" t="s">
-        <v>142</v>
+        <v>275</v>
       </c>
       <c r="C3" s="3" t="s">
-        <v>43</v>
+        <v>54</v>
       </c>
       <c r="D3" s="3" t="s">
-        <v>137</v>
+        <v>270</v>
       </c>
       <c r="E3" s="3" t="s">
-        <v>143</v>
+        <v>276</v>
       </c>
       <c r="F3" s="3" t="s">
-        <v>144</v>
+        <v>277</v>
       </c>
       <c r="G3" s="3" t="s">
-        <v>145</v>
+        <v>278</v>
       </c>
       <c r="H3" s="3" t="s">
-        <v>146</v>
+        <v>279</v>
       </c>
       <c r="I3" s="3"/>
     </row>
     <row r="4" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A4" s="3" t="s">
-        <v>147</v>
+        <v>280</v>
       </c>
       <c r="B4" s="3" t="s">
-        <v>99</v>
+        <v>169</v>
       </c>
       <c r="C4" s="3" t="s">
         <v>27</v>
       </c>
       <c r="D4" s="3" t="s">
-        <v>148</v>
+        <v>281</v>
       </c>
       <c r="E4" s="3" t="s">
-        <v>149</v>
+        <v>282</v>
       </c>
       <c r="F4" s="3"/>
       <c r="G4" s="3" t="s">
-        <v>150</v>
+        <v>283</v>
       </c>
       <c r="H4" s="3" t="s">
-        <v>151</v>
+        <v>284</v>
       </c>
       <c r="I4" s="3"/>
     </row>
     <row r="5" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A5" s="3" t="s">
-        <v>96</v>
+        <v>154</v>
       </c>
       <c r="B5" s="3" t="s">
-        <v>142</v>
+        <v>275</v>
       </c>
       <c r="C5" s="3" t="s">
-        <v>52</v>
+        <v>63</v>
       </c>
       <c r="D5" s="3" t="s">
-        <v>148</v>
+        <v>281</v>
       </c>
       <c r="E5" s="3" t="s">
-        <v>152</v>
+        <v>285</v>
       </c>
       <c r="F5" s="3"/>
       <c r="G5" s="3" t="s">
-        <v>150</v>
+        <v>283</v>
       </c>
       <c r="H5" s="3" t="s">
-        <v>153</v>
+        <v>286</v>
       </c>
       <c r="I5" s="3"/>
     </row>
+    <row r="6" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A6" s="3" t="s">
+        <v>157</v>
+      </c>
+      <c r="B6" s="3" t="s">
+        <v>275</v>
+      </c>
+      <c r="C6" s="3" t="s">
+        <v>70</v>
+      </c>
+      <c r="D6" s="3" t="s">
+        <v>287</v>
+      </c>
+      <c r="E6" s="3" t="s">
+        <v>288</v>
+      </c>
+      <c r="F6" s="3" t="s">
+        <v>289</v>
+      </c>
+      <c r="G6" s="3" t="s">
+        <v>290</v>
+      </c>
+      <c r="H6" s="3" t="s">
+        <v>291</v>
+      </c>
+      <c r="I6" s="3" t="s">
+        <v>292</v>
+      </c>
+    </row>
+    <row r="7" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A7" s="3" t="s">
+        <v>160</v>
+      </c>
+      <c r="B7" s="3" t="s">
+        <v>275</v>
+      </c>
+      <c r="C7" s="3" t="s">
+        <v>80</v>
+      </c>
+      <c r="D7" s="3" t="s">
+        <v>287</v>
+      </c>
+      <c r="E7" s="3" t="s">
+        <v>293</v>
+      </c>
+      <c r="F7" s="3" t="s">
+        <v>294</v>
+      </c>
+      <c r="G7" s="3" t="s">
+        <v>295</v>
+      </c>
+      <c r="H7" s="3" t="s">
+        <v>296</v>
+      </c>
+      <c r="I7" s="3" t="s">
+        <v>292</v>
+      </c>
+    </row>
+    <row r="8" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A8" s="3" t="s">
+        <v>163</v>
+      </c>
+      <c r="B8" s="3" t="s">
+        <v>275</v>
+      </c>
+      <c r="C8" s="3" t="s">
+        <v>89</v>
+      </c>
+      <c r="D8" s="3" t="s">
+        <v>287</v>
+      </c>
+      <c r="E8" s="3" t="s">
+        <v>297</v>
+      </c>
+      <c r="F8" s="3" t="s">
+        <v>298</v>
+      </c>
+      <c r="G8" s="3" t="s">
+        <v>299</v>
+      </c>
+      <c r="H8" s="3" t="s">
+        <v>300</v>
+      </c>
+      <c r="I8" s="3" t="s">
+        <v>292</v>
+      </c>
+    </row>
+    <row r="9" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A9" s="3" t="s">
+        <v>166</v>
+      </c>
+      <c r="B9" s="3" t="s">
+        <v>275</v>
+      </c>
+      <c r="C9" s="3" t="s">
+        <v>96</v>
+      </c>
+      <c r="D9" s="3" t="s">
+        <v>287</v>
+      </c>
+      <c r="E9" s="3" t="s">
+        <v>301</v>
+      </c>
+      <c r="F9" s="3" t="s">
+        <v>302</v>
+      </c>
+      <c r="G9" s="3" t="s">
+        <v>303</v>
+      </c>
+      <c r="H9" s="3" t="s">
+        <v>304</v>
+      </c>
+      <c r="I9" s="3" t="s">
+        <v>292</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:I5"/>
+  <autoFilter ref="A1:I9"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
 </worksheet>
@@ -1691,59 +3151,58 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:M3"/>
+  <dimension ref="A1:M7"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="15" customWidth="1"/>
     <col min="2" max="2" width="12" customWidth="1"/>
     <col min="3" max="3" width="40" customWidth="1"/>
-    <col min="4" max="4" width="12" customWidth="1"/>
-    <col min="5" max="5" width="14" customWidth="1"/>
+    <col min="4" max="5" width="14" customWidth="1"/>
     <col min="6" max="6" width="12" customWidth="1"/>
-    <col min="7" max="7" width="15" customWidth="1"/>
-    <col min="8" max="8" width="13" customWidth="1"/>
-    <col min="9" max="10" width="12" customWidth="1"/>
-    <col min="11" max="11" width="29" customWidth="1"/>
-    <col min="12" max="12" width="40" customWidth="1"/>
+    <col min="7" max="7" width="19" customWidth="1"/>
+    <col min="8" max="8" width="17" customWidth="1"/>
+    <col min="9" max="9" width="25" customWidth="1"/>
+    <col min="10" max="10" width="12" customWidth="1"/>
+    <col min="11" max="12" width="40" customWidth="1"/>
     <col min="13" max="13" width="24" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" ht="24" customHeight="1" spans="1:13" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="2" t="s">
-        <v>31</v>
+        <v>42</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>32</v>
+        <v>43</v>
       </c>
       <c r="C1" s="2" t="s">
-        <v>33</v>
+        <v>44</v>
       </c>
       <c r="D1" s="2" t="s">
-        <v>34</v>
+        <v>45</v>
       </c>
       <c r="E1" s="2" t="s">
-        <v>35</v>
+        <v>46</v>
       </c>
       <c r="F1" s="2" t="s">
-        <v>36</v>
+        <v>47</v>
       </c>
       <c r="G1" s="2" t="s">
-        <v>37</v>
+        <v>48</v>
       </c>
       <c r="H1" s="2" t="s">
-        <v>38</v>
+        <v>49</v>
       </c>
       <c r="I1" s="2" t="s">
-        <v>39</v>
+        <v>50</v>
       </c>
       <c r="J1" s="2" t="s">
-        <v>40</v>
+        <v>51</v>
       </c>
       <c r="K1" s="2" t="s">
-        <v>41</v>
+        <v>52</v>
       </c>
       <c r="L1" s="2" t="s">
-        <v>42</v>
+        <v>53</v>
       </c>
       <c r="M1" s="2" t="s">
         <v>17</v>
@@ -1751,40 +3210,40 @@
     </row>
     <row r="2" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A2" s="3" t="s">
-        <v>43</v>
+        <v>54</v>
       </c>
       <c r="B2" s="3" t="s">
-        <v>44</v>
+        <v>55</v>
       </c>
       <c r="C2" s="3" t="s">
-        <v>45</v>
+        <v>56</v>
       </c>
       <c r="D2" s="3" t="s">
         <v>19</v>
       </c>
       <c r="E2" s="3" t="s">
-        <v>46</v>
+        <v>57</v>
       </c>
       <c r="F2" s="3">
         <v>90</v>
       </c>
       <c r="G2" s="3" t="s">
-        <v>47</v>
+        <v>58</v>
       </c>
       <c r="H2" s="3" t="s">
-        <v>48</v>
+        <v>59</v>
       </c>
       <c r="I2" s="3" t="s">
         <v>22</v>
       </c>
       <c r="J2" s="3" t="s">
-        <v>49</v>
+        <v>60</v>
       </c>
       <c r="K2" s="3" t="s">
-        <v>50</v>
+        <v>61</v>
       </c>
       <c r="L2" s="3" t="s">
-        <v>51</v>
+        <v>62</v>
       </c>
       <c r="M2" s="3" t="s">
         <v>26</v>
@@ -1792,28 +3251,28 @@
     </row>
     <row r="3" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A3" s="3" t="s">
-        <v>52</v>
+        <v>63</v>
       </c>
       <c r="B3" s="3" t="s">
-        <v>53</v>
+        <v>64</v>
       </c>
       <c r="C3" s="3" t="s">
-        <v>54</v>
+        <v>65</v>
       </c>
       <c r="D3" s="3" t="s">
         <v>28</v>
       </c>
       <c r="E3" s="3" t="s">
-        <v>55</v>
+        <v>66</v>
       </c>
       <c r="F3" s="3">
         <v>127</v>
       </c>
       <c r="G3" s="3" t="s">
-        <v>56</v>
+        <v>67</v>
       </c>
       <c r="H3" s="3" t="s">
-        <v>57</v>
+        <v>68</v>
       </c>
       <c r="I3" s="3" t="s">
         <v>22</v>
@@ -1822,7 +3281,7 @@
         <v>22</v>
       </c>
       <c r="K3" s="3" t="s">
-        <v>58</v>
+        <v>69</v>
       </c>
       <c r="L3" s="3" t="s">
         <v>22</v>
@@ -1831,8 +3290,172 @@
         <v>30</v>
       </c>
     </row>
+    <row r="4" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A4" s="3" t="s">
+        <v>70</v>
+      </c>
+      <c r="B4" s="3" t="s">
+        <v>71</v>
+      </c>
+      <c r="C4" s="3" t="s">
+        <v>72</v>
+      </c>
+      <c r="D4" s="3" t="s">
+        <v>73</v>
+      </c>
+      <c r="E4" s="3" t="s">
+        <v>74</v>
+      </c>
+      <c r="F4" s="3">
+        <v>150</v>
+      </c>
+      <c r="G4" s="3" t="s">
+        <v>75</v>
+      </c>
+      <c r="H4" s="3" t="s">
+        <v>76</v>
+      </c>
+      <c r="I4" s="3" t="s">
+        <v>22</v>
+      </c>
+      <c r="J4" s="3" t="s">
+        <v>77</v>
+      </c>
+      <c r="K4" s="3" t="s">
+        <v>78</v>
+      </c>
+      <c r="L4" s="3" t="s">
+        <v>79</v>
+      </c>
+      <c r="M4" s="3" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="5" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A5" s="3" t="s">
+        <v>80</v>
+      </c>
+      <c r="B5" s="3" t="s">
+        <v>81</v>
+      </c>
+      <c r="C5" s="3" t="s">
+        <v>82</v>
+      </c>
+      <c r="D5" s="3" t="s">
+        <v>37</v>
+      </c>
+      <c r="E5" s="3" t="s">
+        <v>83</v>
+      </c>
+      <c r="F5" s="3">
+        <v>150</v>
+      </c>
+      <c r="G5" s="3" t="s">
+        <v>84</v>
+      </c>
+      <c r="H5" s="3" t="s">
+        <v>85</v>
+      </c>
+      <c r="I5" s="3" t="s">
+        <v>22</v>
+      </c>
+      <c r="J5" s="3" t="s">
+        <v>86</v>
+      </c>
+      <c r="K5" s="3" t="s">
+        <v>87</v>
+      </c>
+      <c r="L5" s="3" t="s">
+        <v>88</v>
+      </c>
+      <c r="M5" s="3" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="6" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A6" s="3" t="s">
+        <v>89</v>
+      </c>
+      <c r="B6" s="3" t="s">
+        <v>90</v>
+      </c>
+      <c r="C6" s="3" t="s">
+        <v>91</v>
+      </c>
+      <c r="D6" s="3" t="s">
+        <v>39</v>
+      </c>
+      <c r="E6" s="3" t="s">
+        <v>92</v>
+      </c>
+      <c r="F6" s="3">
+        <v>160</v>
+      </c>
+      <c r="G6" s="3" t="s">
+        <v>67</v>
+      </c>
+      <c r="H6" s="3" t="s">
+        <v>68</v>
+      </c>
+      <c r="I6" s="3" t="s">
+        <v>22</v>
+      </c>
+      <c r="J6" s="3" t="s">
+        <v>93</v>
+      </c>
+      <c r="K6" s="3" t="s">
+        <v>94</v>
+      </c>
+      <c r="L6" s="3" t="s">
+        <v>95</v>
+      </c>
+      <c r="M6" s="3" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="7" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A7" s="3" t="s">
+        <v>96</v>
+      </c>
+      <c r="B7" s="3" t="s">
+        <v>97</v>
+      </c>
+      <c r="C7" s="3" t="s">
+        <v>98</v>
+      </c>
+      <c r="D7" s="3" t="s">
+        <v>41</v>
+      </c>
+      <c r="E7" s="3" t="s">
+        <v>99</v>
+      </c>
+      <c r="F7" s="3">
+        <v>119</v>
+      </c>
+      <c r="G7" s="3" t="s">
+        <v>100</v>
+      </c>
+      <c r="H7" s="3" t="s">
+        <v>101</v>
+      </c>
+      <c r="I7" s="3" t="s">
+        <v>102</v>
+      </c>
+      <c r="J7" s="3" t="s">
+        <v>22</v>
+      </c>
+      <c r="K7" s="3" t="s">
+        <v>103</v>
+      </c>
+      <c r="L7" s="3" t="s">
+        <v>104</v>
+      </c>
+      <c r="M7" s="3" t="s">
+        <v>33</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:M3"/>
+  <autoFilter ref="A1:M7"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
 </worksheet>
@@ -1840,7 +3463,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:T3"/>
+  <dimension ref="A1:T8"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="18" customWidth="1"/>
@@ -1866,7 +3489,7 @@
         <v>3</v>
       </c>
       <c r="E1" s="5" t="s">
-        <v>59</v>
+        <v>105</v>
       </c>
       <c r="F1" s="5" t="s">
         <v>6</v>
@@ -1881,13 +3504,13 @@
         <v>9</v>
       </c>
       <c r="J1" s="5" t="s">
-        <v>60</v>
+        <v>106</v>
       </c>
       <c r="K1" s="5" t="s">
-        <v>61</v>
+        <v>107</v>
       </c>
       <c r="L1" s="5" t="s">
-        <v>62</v>
+        <v>108</v>
       </c>
       <c r="M1" s="5" t="s">
         <v>11</v>
@@ -1908,7 +3531,7 @@
         <v>16</v>
       </c>
       <c r="S1" s="5" t="s">
-        <v>63</v>
+        <v>109</v>
       </c>
       <c r="T1" s="5" t="s">
         <v>17</v>
@@ -1974,7 +3597,7 @@
         <v>29</v>
       </c>
       <c r="E3" s="3" t="s">
-        <v>64</v>
+        <v>110</v>
       </c>
       <c r="F3" s="3"/>
       <c r="G3" s="3"/>
@@ -1996,8 +3619,178 @@
         <v>30</v>
       </c>
     </row>
+    <row r="4" spans="1:20" x14ac:dyDescent="0.25">
+      <c r="A4" s="3" t="s">
+        <v>31</v>
+      </c>
+      <c r="B4" s="3" t="s">
+        <v>32</v>
+      </c>
+      <c r="C4" s="3" t="s">
+        <v>32</v>
+      </c>
+      <c r="D4" s="3"/>
+      <c r="E4" s="3"/>
+      <c r="F4" s="3"/>
+      <c r="G4" s="3"/>
+      <c r="H4" s="3"/>
+      <c r="I4" s="3"/>
+      <c r="J4" s="3"/>
+      <c r="K4" s="3"/>
+      <c r="L4" s="3"/>
+      <c r="M4" s="3"/>
+      <c r="N4" s="3"/>
+      <c r="O4" s="3"/>
+      <c r="P4" s="3" t="s">
+        <v>21</v>
+      </c>
+      <c r="Q4" s="3"/>
+      <c r="R4" s="3"/>
+      <c r="S4" s="3" t="s">
+        <v>33</v>
+      </c>
+      <c r="T4" s="3" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="5" spans="1:20" x14ac:dyDescent="0.25">
+      <c r="A5" s="3" t="s">
+        <v>34</v>
+      </c>
+      <c r="B5" s="3" t="s">
+        <v>35</v>
+      </c>
+      <c r="C5" s="3" t="s">
+        <v>35</v>
+      </c>
+      <c r="D5" s="3"/>
+      <c r="E5" s="3"/>
+      <c r="F5" s="3"/>
+      <c r="G5" s="3"/>
+      <c r="H5" s="3"/>
+      <c r="I5" s="3"/>
+      <c r="J5" s="3"/>
+      <c r="K5" s="3"/>
+      <c r="L5" s="3"/>
+      <c r="M5" s="3"/>
+      <c r="N5" s="3"/>
+      <c r="O5" s="3"/>
+      <c r="P5" s="3" t="s">
+        <v>21</v>
+      </c>
+      <c r="Q5" s="3"/>
+      <c r="R5" s="3"/>
+      <c r="S5" s="3" t="s">
+        <v>33</v>
+      </c>
+      <c r="T5" s="3" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="6" spans="1:20" x14ac:dyDescent="0.25">
+      <c r="A6" s="3" t="s">
+        <v>36</v>
+      </c>
+      <c r="B6" s="3" t="s">
+        <v>37</v>
+      </c>
+      <c r="C6" s="3"/>
+      <c r="D6" s="3" t="s">
+        <v>37</v>
+      </c>
+      <c r="E6" s="3"/>
+      <c r="F6" s="3"/>
+      <c r="G6" s="3"/>
+      <c r="H6" s="3"/>
+      <c r="I6" s="3"/>
+      <c r="J6" s="3"/>
+      <c r="K6" s="3"/>
+      <c r="L6" s="3"/>
+      <c r="M6" s="3"/>
+      <c r="N6" s="3"/>
+      <c r="O6" s="3"/>
+      <c r="P6" s="3" t="s">
+        <v>21</v>
+      </c>
+      <c r="Q6" s="3"/>
+      <c r="R6" s="3"/>
+      <c r="S6" s="3" t="s">
+        <v>33</v>
+      </c>
+      <c r="T6" s="3" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="7" spans="1:20" x14ac:dyDescent="0.25">
+      <c r="A7" s="3" t="s">
+        <v>38</v>
+      </c>
+      <c r="B7" s="3" t="s">
+        <v>39</v>
+      </c>
+      <c r="C7" s="3" t="s">
+        <v>39</v>
+      </c>
+      <c r="D7" s="3"/>
+      <c r="E7" s="3"/>
+      <c r="F7" s="3"/>
+      <c r="G7" s="3"/>
+      <c r="H7" s="3"/>
+      <c r="I7" s="3"/>
+      <c r="J7" s="3"/>
+      <c r="K7" s="3"/>
+      <c r="L7" s="3"/>
+      <c r="M7" s="3"/>
+      <c r="N7" s="3"/>
+      <c r="O7" s="3"/>
+      <c r="P7" s="3" t="s">
+        <v>21</v>
+      </c>
+      <c r="Q7" s="3"/>
+      <c r="R7" s="3"/>
+      <c r="S7" s="3" t="s">
+        <v>33</v>
+      </c>
+      <c r="T7" s="3" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="8" spans="1:20" x14ac:dyDescent="0.25">
+      <c r="A8" s="3" t="s">
+        <v>40</v>
+      </c>
+      <c r="B8" s="3" t="s">
+        <v>41</v>
+      </c>
+      <c r="C8" s="3" t="s">
+        <v>41</v>
+      </c>
+      <c r="D8" s="3"/>
+      <c r="E8" s="3"/>
+      <c r="F8" s="3"/>
+      <c r="G8" s="3"/>
+      <c r="H8" s="3"/>
+      <c r="I8" s="3"/>
+      <c r="J8" s="3"/>
+      <c r="K8" s="3"/>
+      <c r="L8" s="3"/>
+      <c r="M8" s="3"/>
+      <c r="N8" s="3"/>
+      <c r="O8" s="3"/>
+      <c r="P8" s="3" t="s">
+        <v>21</v>
+      </c>
+      <c r="Q8" s="3"/>
+      <c r="R8" s="3"/>
+      <c r="S8" s="3" t="s">
+        <v>33</v>
+      </c>
+      <c r="T8" s="3" t="s">
+        <v>33</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:T3"/>
+  <autoFilter ref="A1:T8"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
 </worksheet>
@@ -2018,7 +3811,7 @@
   <sheetData>
     <row r="1" ht="24" customHeight="1" spans="1:8" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="5" t="s">
-        <v>65</v>
+        <v>111</v>
       </c>
       <c r="B1" s="5" t="s">
         <v>0</v>
@@ -2027,24 +3820,24 @@
         <v>4</v>
       </c>
       <c r="D1" s="5" t="s">
-        <v>66</v>
+        <v>112</v>
       </c>
       <c r="E1" s="5" t="s">
-        <v>67</v>
+        <v>113</v>
       </c>
       <c r="F1" s="5" t="s">
-        <v>68</v>
+        <v>114</v>
       </c>
       <c r="G1" s="5" t="s">
-        <v>69</v>
+        <v>115</v>
       </c>
       <c r="H1" s="5" t="s">
-        <v>63</v>
+        <v>109</v>
       </c>
     </row>
     <row r="2" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A2" s="3" t="s">
-        <v>70</v>
+        <v>116</v>
       </c>
       <c r="B2" s="3" t="s">
         <v>18</v>
@@ -2053,10 +3846,10 @@
         <v>20</v>
       </c>
       <c r="D2" s="3" t="s">
-        <v>71</v>
+        <v>117</v>
       </c>
       <c r="E2" s="3" t="s">
-        <v>72</v>
+        <v>118</v>
       </c>
       <c r="F2" s="3" t="b">
         <v>0</v>
@@ -2075,7 +3868,7 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:P3"/>
+  <dimension ref="A1:P7"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="15" customWidth="1"/>
@@ -2084,57 +3877,58 @@
     <col min="5" max="5" width="14" customWidth="1"/>
     <col min="6" max="6" width="12" customWidth="1"/>
     <col min="7" max="8" width="16" customWidth="1"/>
-    <col min="9" max="10" width="12" customWidth="1"/>
-    <col min="11" max="11" width="40" customWidth="1"/>
-    <col min="12" max="14" width="12" customWidth="1"/>
+    <col min="9" max="9" width="17" customWidth="1"/>
+    <col min="10" max="10" width="12" customWidth="1"/>
+    <col min="11" max="12" width="40" customWidth="1"/>
+    <col min="13" max="14" width="12" customWidth="1"/>
     <col min="15" max="16" width="24" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" ht="24" customHeight="1" spans="1:16" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="5" t="s">
-        <v>31</v>
+        <v>42</v>
       </c>
       <c r="B1" s="5" t="s">
-        <v>73</v>
+        <v>119</v>
       </c>
       <c r="C1" s="5" t="s">
-        <v>74</v>
+        <v>120</v>
       </c>
       <c r="D1" s="5" t="s">
-        <v>33</v>
+        <v>44</v>
       </c>
       <c r="E1" s="5" t="s">
-        <v>35</v>
+        <v>46</v>
       </c>
       <c r="F1" s="5" t="s">
-        <v>36</v>
+        <v>47</v>
       </c>
       <c r="G1" s="5" t="s">
-        <v>75</v>
+        <v>121</v>
       </c>
       <c r="H1" s="5" t="s">
-        <v>76</v>
+        <v>122</v>
       </c>
       <c r="I1" s="5" t="s">
-        <v>77</v>
+        <v>123</v>
       </c>
       <c r="J1" s="5" t="s">
         <v>16</v>
       </c>
       <c r="K1" s="5" t="s">
-        <v>42</v>
+        <v>53</v>
       </c>
       <c r="L1" s="5" t="s">
-        <v>78</v>
+        <v>124</v>
       </c>
       <c r="M1" s="5" t="s">
-        <v>79</v>
+        <v>125</v>
       </c>
       <c r="N1" s="5" t="s">
-        <v>80</v>
+        <v>126</v>
       </c>
       <c r="O1" s="5" t="s">
-        <v>63</v>
+        <v>109</v>
       </c>
       <c r="P1" s="5" t="s">
         <v>17</v>
@@ -2142,33 +3936,33 @@
     </row>
     <row r="2" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A2" s="3" t="s">
-        <v>43</v>
+        <v>54</v>
       </c>
       <c r="B2" s="3" t="s">
-        <v>44</v>
+        <v>55</v>
       </c>
       <c r="C2" s="3" t="s">
-        <v>45</v>
+        <v>56</v>
       </c>
       <c r="D2" s="3" t="s">
-        <v>45</v>
+        <v>56</v>
       </c>
       <c r="E2" s="3" t="s">
-        <v>46</v>
+        <v>57</v>
       </c>
       <c r="F2" s="3">
         <v>90</v>
       </c>
       <c r="G2" s="3" t="s">
-        <v>81</v>
+        <v>127</v>
       </c>
       <c r="H2" s="3" t="s">
-        <v>82</v>
+        <v>128</v>
       </c>
       <c r="I2" s="3"/>
       <c r="J2" s="3"/>
       <c r="K2" s="3" t="s">
-        <v>51</v>
+        <v>62</v>
       </c>
       <c r="L2" s="3"/>
       <c r="M2" s="3"/>
@@ -2182,28 +3976,28 @@
     </row>
     <row r="3" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A3" s="3" t="s">
-        <v>52</v>
+        <v>63</v>
       </c>
       <c r="B3" s="3" t="s">
-        <v>53</v>
+        <v>64</v>
       </c>
       <c r="C3" s="3" t="s">
-        <v>83</v>
+        <v>129</v>
       </c>
       <c r="D3" s="3" t="s">
-        <v>54</v>
+        <v>65</v>
       </c>
       <c r="E3" s="3" t="s">
-        <v>55</v>
+        <v>66</v>
       </c>
       <c r="F3" s="3">
         <v>127</v>
       </c>
       <c r="G3" s="3" t="s">
-        <v>84</v>
+        <v>130</v>
       </c>
       <c r="H3" s="3" t="s">
-        <v>85</v>
+        <v>131</v>
       </c>
       <c r="I3" s="3"/>
       <c r="J3" s="3"/>
@@ -2218,8 +4012,186 @@
         <v>30</v>
       </c>
     </row>
+    <row r="4" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A4" s="3" t="s">
+        <v>70</v>
+      </c>
+      <c r="B4" s="3" t="s">
+        <v>71</v>
+      </c>
+      <c r="C4" s="3" t="s">
+        <v>72</v>
+      </c>
+      <c r="D4" s="3" t="s">
+        <v>72</v>
+      </c>
+      <c r="E4" s="3" t="s">
+        <v>74</v>
+      </c>
+      <c r="F4" s="3">
+        <v>150</v>
+      </c>
+      <c r="G4" s="3" t="s">
+        <v>132</v>
+      </c>
+      <c r="H4" s="3" t="s">
+        <v>133</v>
+      </c>
+      <c r="I4" s="3"/>
+      <c r="J4" s="3"/>
+      <c r="K4" s="3" t="s">
+        <v>79</v>
+      </c>
+      <c r="L4" s="3" t="s">
+        <v>134</v>
+      </c>
+      <c r="M4" s="3"/>
+      <c r="N4" s="3" t="s">
+        <v>135</v>
+      </c>
+      <c r="O4" s="3" t="s">
+        <v>33</v>
+      </c>
+      <c r="P4" s="3" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="5" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A5" s="3" t="s">
+        <v>80</v>
+      </c>
+      <c r="B5" s="3" t="s">
+        <v>81</v>
+      </c>
+      <c r="C5" s="3" t="s">
+        <v>82</v>
+      </c>
+      <c r="D5" s="3" t="s">
+        <v>82</v>
+      </c>
+      <c r="E5" s="3" t="s">
+        <v>83</v>
+      </c>
+      <c r="F5" s="3">
+        <v>150</v>
+      </c>
+      <c r="G5" s="3" t="s">
+        <v>136</v>
+      </c>
+      <c r="H5" s="3" t="s">
+        <v>137</v>
+      </c>
+      <c r="I5" s="3"/>
+      <c r="J5" s="3"/>
+      <c r="K5" s="3" t="s">
+        <v>88</v>
+      </c>
+      <c r="L5" s="3" t="s">
+        <v>138</v>
+      </c>
+      <c r="M5" s="3"/>
+      <c r="N5" s="3" t="s">
+        <v>135</v>
+      </c>
+      <c r="O5" s="3" t="s">
+        <v>33</v>
+      </c>
+      <c r="P5" s="3" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="6" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A6" s="3" t="s">
+        <v>89</v>
+      </c>
+      <c r="B6" s="3" t="s">
+        <v>90</v>
+      </c>
+      <c r="C6" s="3" t="s">
+        <v>91</v>
+      </c>
+      <c r="D6" s="3" t="s">
+        <v>91</v>
+      </c>
+      <c r="E6" s="3" t="s">
+        <v>92</v>
+      </c>
+      <c r="F6" s="3">
+        <v>160</v>
+      </c>
+      <c r="G6" s="3" t="s">
+        <v>130</v>
+      </c>
+      <c r="H6" s="3" t="s">
+        <v>131</v>
+      </c>
+      <c r="I6" s="3"/>
+      <c r="J6" s="3"/>
+      <c r="K6" s="3" t="s">
+        <v>95</v>
+      </c>
+      <c r="L6" s="3" t="s">
+        <v>139</v>
+      </c>
+      <c r="M6" s="3"/>
+      <c r="N6" s="3" t="s">
+        <v>135</v>
+      </c>
+      <c r="O6" s="3" t="s">
+        <v>33</v>
+      </c>
+      <c r="P6" s="3" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="7" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A7" s="3" t="s">
+        <v>96</v>
+      </c>
+      <c r="B7" s="3" t="s">
+        <v>97</v>
+      </c>
+      <c r="C7" s="3" t="s">
+        <v>98</v>
+      </c>
+      <c r="D7" s="3" t="s">
+        <v>98</v>
+      </c>
+      <c r="E7" s="3" t="s">
+        <v>99</v>
+      </c>
+      <c r="F7" s="3">
+        <v>119</v>
+      </c>
+      <c r="G7" s="3" t="s">
+        <v>140</v>
+      </c>
+      <c r="H7" s="3" t="s">
+        <v>141</v>
+      </c>
+      <c r="I7" s="3" t="s">
+        <v>142</v>
+      </c>
+      <c r="J7" s="3"/>
+      <c r="K7" s="3" t="s">
+        <v>104</v>
+      </c>
+      <c r="L7" s="3" t="s">
+        <v>143</v>
+      </c>
+      <c r="M7" s="3"/>
+      <c r="N7" s="3" t="s">
+        <v>135</v>
+      </c>
+      <c r="O7" s="3" t="s">
+        <v>33</v>
+      </c>
+      <c r="P7" s="3" t="s">
+        <v>33</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:P3"/>
+  <autoFilter ref="A1:P7"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
 </worksheet>
@@ -2227,7 +4199,7 @@
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:G3"/>
+  <dimension ref="A1:G7"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="2" width="15" customWidth="1"/>
@@ -2237,75 +4209,167 @@
   <sheetData>
     <row r="1" ht="24" customHeight="1" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="5" t="s">
-        <v>86</v>
+        <v>144</v>
       </c>
       <c r="B1" s="5" t="s">
-        <v>31</v>
+        <v>42</v>
       </c>
       <c r="C1" s="5" t="s">
-        <v>32</v>
+        <v>43</v>
       </c>
       <c r="D1" s="5" t="s">
-        <v>87</v>
+        <v>145</v>
       </c>
       <c r="E1" s="5" t="s">
-        <v>88</v>
+        <v>146</v>
       </c>
       <c r="F1" s="5" t="s">
-        <v>89</v>
+        <v>147</v>
       </c>
       <c r="G1" s="5" t="s">
-        <v>69</v>
+        <v>115</v>
       </c>
     </row>
     <row r="2" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A2" s="3" t="s">
-        <v>90</v>
+        <v>148</v>
       </c>
       <c r="B2" s="3" t="s">
-        <v>43</v>
+        <v>54</v>
       </c>
       <c r="C2" s="3" t="s">
-        <v>44</v>
+        <v>55</v>
       </c>
       <c r="D2" s="3" t="s">
-        <v>91</v>
+        <v>149</v>
       </c>
       <c r="E2" s="3" t="s">
-        <v>92</v>
+        <v>150</v>
       </c>
       <c r="F2" s="3" t="b">
         <v>1</v>
       </c>
       <c r="G2" s="3" t="s">
-        <v>93</v>
+        <v>151</v>
       </c>
     </row>
     <row r="3" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A3" s="3" t="s">
-        <v>94</v>
+        <v>152</v>
       </c>
       <c r="B3" s="3" t="s">
-        <v>52</v>
+        <v>63</v>
       </c>
       <c r="C3" s="3" t="s">
-        <v>53</v>
+        <v>64</v>
       </c>
       <c r="D3" s="3" t="s">
-        <v>95</v>
+        <v>153</v>
       </c>
       <c r="E3" s="3" t="s">
-        <v>92</v>
+        <v>150</v>
       </c>
       <c r="F3" s="3" t="b">
         <v>1</v>
       </c>
       <c r="G3" s="3" t="s">
+        <v>154</v>
+      </c>
+    </row>
+    <row r="4" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A4" s="3" t="s">
+        <v>155</v>
+      </c>
+      <c r="B4" s="3" t="s">
+        <v>70</v>
+      </c>
+      <c r="C4" s="3" t="s">
+        <v>71</v>
+      </c>
+      <c r="D4" s="3" t="s">
+        <v>156</v>
+      </c>
+      <c r="E4" s="3" t="s">
+        <v>150</v>
+      </c>
+      <c r="F4" s="3" t="b">
+        <v>1</v>
+      </c>
+      <c r="G4" s="3" t="s">
+        <v>157</v>
+      </c>
+    </row>
+    <row r="5" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A5" s="3" t="s">
+        <v>158</v>
+      </c>
+      <c r="B5" s="3" t="s">
+        <v>80</v>
+      </c>
+      <c r="C5" s="3" t="s">
+        <v>81</v>
+      </c>
+      <c r="D5" s="3" t="s">
+        <v>159</v>
+      </c>
+      <c r="E5" s="3" t="s">
+        <v>150</v>
+      </c>
+      <c r="F5" s="3" t="b">
+        <v>1</v>
+      </c>
+      <c r="G5" s="3" t="s">
+        <v>160</v>
+      </c>
+    </row>
+    <row r="6" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A6" s="3" t="s">
+        <v>161</v>
+      </c>
+      <c r="B6" s="3" t="s">
+        <v>89</v>
+      </c>
+      <c r="C6" s="3" t="s">
+        <v>90</v>
+      </c>
+      <c r="D6" s="3" t="s">
+        <v>162</v>
+      </c>
+      <c r="E6" s="3" t="s">
+        <v>150</v>
+      </c>
+      <c r="F6" s="3" t="b">
+        <v>1</v>
+      </c>
+      <c r="G6" s="3" t="s">
+        <v>163</v>
+      </c>
+    </row>
+    <row r="7" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A7" s="3" t="s">
+        <v>164</v>
+      </c>
+      <c r="B7" s="3" t="s">
         <v>96</v>
       </c>
+      <c r="C7" s="3" t="s">
+        <v>97</v>
+      </c>
+      <c r="D7" s="3" t="s">
+        <v>165</v>
+      </c>
+      <c r="E7" s="3" t="s">
+        <v>150</v>
+      </c>
+      <c r="F7" s="3" t="b">
+        <v>1</v>
+      </c>
+      <c r="G7" s="3" t="s">
+        <v>166</v>
+      </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:G3"/>
+  <autoFilter ref="A1:G7"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
 </worksheet>
@@ -2313,7 +4377,7 @@
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:D3"/>
+  <dimension ref="A1:D8"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="15" customWidth="1"/>
@@ -2323,27 +4387,27 @@
   <sheetData>
     <row r="1" ht="24" customHeight="1" spans="1:4" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="5" t="s">
-        <v>31</v>
+        <v>42</v>
       </c>
       <c r="B1" s="5" t="s">
         <v>0</v>
       </c>
       <c r="C1" s="5" t="s">
-        <v>97</v>
+        <v>167</v>
       </c>
       <c r="D1" s="5" t="s">
-        <v>98</v>
+        <v>168</v>
       </c>
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A2" s="3" t="s">
-        <v>43</v>
+        <v>54</v>
       </c>
       <c r="B2" s="3" t="s">
         <v>18</v>
       </c>
       <c r="C2" s="3" t="s">
-        <v>99</v>
+        <v>169</v>
       </c>
       <c r="D2" s="3">
         <v>1</v>
@@ -2351,20 +4415,90 @@
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A3" s="3" t="s">
-        <v>52</v>
+        <v>63</v>
       </c>
       <c r="B3" s="3" t="s">
         <v>27</v>
       </c>
       <c r="C3" s="3" t="s">
-        <v>99</v>
+        <v>169</v>
       </c>
       <c r="D3" s="3">
         <v>1</v>
       </c>
     </row>
+    <row r="4" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A4" s="3" t="s">
+        <v>70</v>
+      </c>
+      <c r="B4" s="3" t="s">
+        <v>31</v>
+      </c>
+      <c r="C4" s="3" t="s">
+        <v>169</v>
+      </c>
+      <c r="D4" s="3">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="5" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A5" s="3" t="s">
+        <v>70</v>
+      </c>
+      <c r="B5" s="3" t="s">
+        <v>34</v>
+      </c>
+      <c r="C5" s="3" t="s">
+        <v>169</v>
+      </c>
+      <c r="D5" s="3">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="6" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A6" s="3" t="s">
+        <v>80</v>
+      </c>
+      <c r="B6" s="3" t="s">
+        <v>36</v>
+      </c>
+      <c r="C6" s="3" t="s">
+        <v>169</v>
+      </c>
+      <c r="D6" s="3">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="7" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A7" s="3" t="s">
+        <v>89</v>
+      </c>
+      <c r="B7" s="3" t="s">
+        <v>38</v>
+      </c>
+      <c r="C7" s="3" t="s">
+        <v>169</v>
+      </c>
+      <c r="D7" s="3">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="8" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A8" s="3" t="s">
+        <v>96</v>
+      </c>
+      <c r="B8" s="3" t="s">
+        <v>40</v>
+      </c>
+      <c r="C8" s="3" t="s">
+        <v>169</v>
+      </c>
+      <c r="D8" s="3">
+        <v>1</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:D3"/>
+  <autoFilter ref="A1:D8"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
 </worksheet>
@@ -2372,7 +4506,7 @@
 
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:B8"/>
+  <dimension ref="A1:B42"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="15" customWidth="1"/>
@@ -2381,70 +4515,342 @@
   <sheetData>
     <row r="1" ht="24" customHeight="1" spans="1:2" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="5" t="s">
-        <v>31</v>
+        <v>42</v>
       </c>
       <c r="B1" s="5" t="s">
-        <v>100</v>
+        <v>170</v>
       </c>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A2" s="3" t="s">
-        <v>43</v>
+        <v>54</v>
       </c>
       <c r="B2" s="3" t="s">
-        <v>101</v>
+        <v>171</v>
       </c>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A3" s="3" t="s">
-        <v>43</v>
+        <v>54</v>
       </c>
       <c r="B3" s="3" t="s">
-        <v>102</v>
+        <v>172</v>
       </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4" s="3" t="s">
-        <v>43</v>
+        <v>54</v>
       </c>
       <c r="B4" s="3" t="s">
-        <v>103</v>
+        <v>173</v>
       </c>
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A5" s="3" t="s">
-        <v>43</v>
+        <v>54</v>
       </c>
       <c r="B5" s="3" t="s">
-        <v>104</v>
+        <v>174</v>
       </c>
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A6" s="3" t="s">
-        <v>43</v>
+        <v>54</v>
       </c>
       <c r="B6" s="3" t="s">
-        <v>105</v>
+        <v>175</v>
       </c>
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A7" s="3" t="s">
-        <v>43</v>
+        <v>54</v>
       </c>
       <c r="B7" s="3" t="s">
-        <v>106</v>
+        <v>176</v>
       </c>
     </row>
     <row r="8" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A8" s="3" t="s">
-        <v>52</v>
+        <v>63</v>
       </c>
       <c r="B8" s="3" t="s">
-        <v>107</v>
+        <v>177</v>
+      </c>
+    </row>
+    <row r="9" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A9" s="3" t="s">
+        <v>70</v>
+      </c>
+      <c r="B9" s="3" t="s">
+        <v>178</v>
+      </c>
+    </row>
+    <row r="10" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A10" s="3" t="s">
+        <v>70</v>
+      </c>
+      <c r="B10" s="3" t="s">
+        <v>174</v>
+      </c>
+    </row>
+    <row r="11" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A11" s="3" t="s">
+        <v>70</v>
+      </c>
+      <c r="B11" s="3" t="s">
+        <v>179</v>
+      </c>
+    </row>
+    <row r="12" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A12" s="3" t="s">
+        <v>70</v>
+      </c>
+      <c r="B12" s="3" t="s">
+        <v>180</v>
+      </c>
+    </row>
+    <row r="13" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A13" s="3" t="s">
+        <v>70</v>
+      </c>
+      <c r="B13" s="3" t="s">
+        <v>181</v>
+      </c>
+    </row>
+    <row r="14" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A14" s="3" t="s">
+        <v>70</v>
+      </c>
+      <c r="B14" s="3" t="s">
+        <v>182</v>
+      </c>
+    </row>
+    <row r="15" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A15" s="3" t="s">
+        <v>70</v>
+      </c>
+      <c r="B15" s="3" t="s">
+        <v>183</v>
+      </c>
+    </row>
+    <row r="16" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A16" s="3" t="s">
+        <v>70</v>
+      </c>
+      <c r="B16" s="3" t="s">
+        <v>184</v>
+      </c>
+    </row>
+    <row r="17" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A17" s="3" t="s">
+        <v>80</v>
+      </c>
+      <c r="B17" s="3" t="s">
+        <v>185</v>
+      </c>
+    </row>
+    <row r="18" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A18" s="3" t="s">
+        <v>80</v>
+      </c>
+      <c r="B18" s="3" t="s">
+        <v>186</v>
+      </c>
+    </row>
+    <row r="19" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A19" s="3" t="s">
+        <v>80</v>
+      </c>
+      <c r="B19" s="3" t="s">
+        <v>173</v>
+      </c>
+    </row>
+    <row r="20" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A20" s="3" t="s">
+        <v>80</v>
+      </c>
+      <c r="B20" s="3" t="s">
+        <v>187</v>
+      </c>
+    </row>
+    <row r="21" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A21" s="3" t="s">
+        <v>80</v>
+      </c>
+      <c r="B21" s="3" t="s">
+        <v>181</v>
+      </c>
+    </row>
+    <row r="22" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A22" s="3" t="s">
+        <v>80</v>
+      </c>
+      <c r="B22" s="3" t="s">
+        <v>188</v>
+      </c>
+    </row>
+    <row r="23" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A23" s="3" t="s">
+        <v>80</v>
+      </c>
+      <c r="B23" s="3" t="s">
+        <v>189</v>
+      </c>
+    </row>
+    <row r="24" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A24" s="3" t="s">
+        <v>80</v>
+      </c>
+      <c r="B24" s="3" t="s">
+        <v>190</v>
+      </c>
+    </row>
+    <row r="25" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A25" s="3" t="s">
+        <v>80</v>
+      </c>
+      <c r="B25" s="3" t="s">
+        <v>184</v>
+      </c>
+    </row>
+    <row r="26" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A26" s="3" t="s">
+        <v>89</v>
+      </c>
+      <c r="B26" s="3" t="s">
+        <v>191</v>
+      </c>
+    </row>
+    <row r="27" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A27" s="3" t="s">
+        <v>89</v>
+      </c>
+      <c r="B27" s="3" t="s">
+        <v>174</v>
+      </c>
+    </row>
+    <row r="28" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A28" s="3" t="s">
+        <v>89</v>
+      </c>
+      <c r="B28" s="3" t="s">
+        <v>186</v>
+      </c>
+    </row>
+    <row r="29" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A29" s="3" t="s">
+        <v>89</v>
+      </c>
+      <c r="B29" s="3" t="s">
+        <v>192</v>
+      </c>
+    </row>
+    <row r="30" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A30" s="3" t="s">
+        <v>89</v>
+      </c>
+      <c r="B30" s="3" t="s">
+        <v>181</v>
+      </c>
+    </row>
+    <row r="31" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A31" s="3" t="s">
+        <v>89</v>
+      </c>
+      <c r="B31" s="3" t="s">
+        <v>193</v>
+      </c>
+    </row>
+    <row r="32" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A32" s="3" t="s">
+        <v>89</v>
+      </c>
+      <c r="B32" s="3" t="s">
+        <v>189</v>
+      </c>
+    </row>
+    <row r="33" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A33" s="3" t="s">
+        <v>89</v>
+      </c>
+      <c r="B33" s="3" t="s">
+        <v>190</v>
+      </c>
+    </row>
+    <row r="34" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A34" s="3" t="s">
+        <v>89</v>
+      </c>
+      <c r="B34" s="3" t="s">
+        <v>184</v>
+      </c>
+    </row>
+    <row r="35" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A35" s="3" t="s">
+        <v>96</v>
+      </c>
+      <c r="B35" s="3" t="s">
+        <v>194</v>
+      </c>
+    </row>
+    <row r="36" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A36" s="3" t="s">
+        <v>96</v>
+      </c>
+      <c r="B36" s="3" t="s">
+        <v>195</v>
+      </c>
+    </row>
+    <row r="37" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A37" s="3" t="s">
+        <v>96</v>
+      </c>
+      <c r="B37" s="3" t="s">
+        <v>196</v>
+      </c>
+    </row>
+    <row r="38" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A38" s="3" t="s">
+        <v>96</v>
+      </c>
+      <c r="B38" s="3" t="s">
+        <v>181</v>
+      </c>
+    </row>
+    <row r="39" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A39" s="3" t="s">
+        <v>96</v>
+      </c>
+      <c r="B39" s="3" t="s">
+        <v>189</v>
+      </c>
+    </row>
+    <row r="40" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A40" s="3" t="s">
+        <v>96</v>
+      </c>
+      <c r="B40" s="3" t="s">
+        <v>190</v>
+      </c>
+    </row>
+    <row r="41" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A41" s="3" t="s">
+        <v>96</v>
+      </c>
+      <c r="B41" s="3" t="s">
+        <v>184</v>
+      </c>
+    </row>
+    <row r="42" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A42" s="3" t="s">
+        <v>96</v>
+      </c>
+      <c r="B42" s="3" t="s">
+        <v>197</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:B8"/>
+  <autoFilter ref="A1:B42"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
 </worksheet>
@@ -2452,7 +4858,7 @@
 
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:C2"/>
+  <dimension ref="A1:C5"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="15" customWidth="1"/>
@@ -2462,28 +4868,61 @@
   <sheetData>
     <row r="1" ht="24" customHeight="1" spans="1:3" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="5" t="s">
-        <v>31</v>
+        <v>42</v>
       </c>
       <c r="B1" s="5" t="s">
-        <v>108</v>
+        <v>198</v>
       </c>
       <c r="C1" s="5" t="s">
-        <v>98</v>
+        <v>168</v>
       </c>
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" s="3" t="s">
-        <v>43</v>
+        <v>54</v>
       </c>
       <c r="B2" s="3" t="s">
-        <v>109</v>
+        <v>199</v>
       </c>
       <c r="C2" s="3">
         <v>1</v>
       </c>
     </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A3" s="3" t="s">
+        <v>70</v>
+      </c>
+      <c r="B3" s="3" t="s">
+        <v>200</v>
+      </c>
+      <c r="C3" s="3">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A4" s="3" t="s">
+        <v>80</v>
+      </c>
+      <c r="B4" s="3" t="s">
+        <v>201</v>
+      </c>
+      <c r="C4" s="3">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A5" s="3" t="s">
+        <v>89</v>
+      </c>
+      <c r="B5" s="3" t="s">
+        <v>202</v>
+      </c>
+      <c r="C5" s="3">
+        <v>1</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:C2"/>
+  <autoFilter ref="A1:C5"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
 </worksheet>

</xml_diff>